<commit_message>
Cover V1: beetle-shaped lattice back shell with ridge crest
- slarc_cover_v1.py: gabled roof (40 deg) with ridge crest, honeycomb
  lattice, side windows, Pi port windows, cable notches, 8 posts on the
  plate column positions (M3 inserts, column screws M3x50 from below),
  inner frames, split at x=-15 with 3x M3. Two parts, printable without
  supports.
- Assembly macro: COVER flag inserts the shell
- BOM + README updated

Checked in FreeCAD: both parts valid single solids, no overlap with Pi
(+HAT envelope), driver, DC-DC, module spots, camera mount, servos;
base fully on plate material.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1771,12 +1771,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Zylinderschraube M3x50</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Säulen obere/untere Platte</t>
+          <t>Säulen obere/untere Platte, von unten in den Gewindeeinsatz des Panzers (ohne Panzer: M3x45 + Mutter)</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -1808,12 +1808,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>unten in den 8 Panzersäulen</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -1845,19 +1845,19 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Säulen + Stoß + Relais</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G33" s="3">
         <f>E33+F33</f>
@@ -1882,19 +1882,19 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G34" s="3">
         <f>E34+F34</f>
@@ -1919,19 +1919,19 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4)</t>
+          <t>Säulen + Stoß + Relais</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G35" s="3">
         <f>E35+F35</f>
@@ -1956,19 +1956,19 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Zylinderschraube M3x14</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F36" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G36" s="3">
         <f>E36+F36</f>
@@ -1993,19 +1993,19 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4)</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F37" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F37" s="7" t="n">
-        <v>1</v>
       </c>
       <c r="G37" s="3">
         <f>E37+F37</f>
@@ -2030,19 +2030,19 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+          <t>Zylinderschraube M2x6</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Pi 5 (M2 geht mit Scheiben)</t>
+          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="3">
         <f>E38+F38</f>
@@ -2067,19 +2067,19 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+          <t>Zylinderschraube M2x25 + Mutter</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" s="3">
         <f>E39+F39</f>
@@ -2104,19 +2104,19 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>für die Distanzbolzen, je 2</t>
+          <t>Pi 5 (M2 geht mit Scheiben)</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="3">
         <f>E40+F40</f>
@@ -2141,12 +2141,16 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr"/>
+          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+        </is>
+      </c>
       <c r="E41" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F41" s="7" t="n">
         <v>0</v>
@@ -2174,19 +2178,19 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
+          <t>Zylinderschraube M2,5x5</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
+          <t>für die Distanzbolzen, je 2</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G42" s="3">
         <f>E42+F42</f>
@@ -2206,21 +2210,17 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>Kabelösen Femur/Tibia</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr"/>
       <c r="E43" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F43" s="7" t="n">
         <v>0</v>
@@ -2243,17 +2243,17 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
@@ -2285,16 +2285,16 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F45" s="7" t="n">
         <v>0</v>
@@ -2322,12 +2322,12 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
@@ -2354,21 +2354,21 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="7" t="n">
         <v>0</v>
@@ -2391,21 +2391,21 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="F48" s="7" t="n">
         <v>0</v>
@@ -2433,16 +2433,16 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>PLA orange (kg)</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="F49" s="7" t="n">
         <v>0</v>
@@ -2460,37 +2460,78 @@
       <c r="K49" s="10" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="n"/>
-      <c r="B50" s="3" t="n"/>
-      <c r="C50" s="3" t="n"/>
-      <c r="D50" s="3" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n"/>
-      <c r="G50" s="3" t="n"/>
-      <c r="H50" s="3" t="n"/>
-      <c r="I50" s="3" t="n"/>
-      <c r="J50" s="3" t="n"/>
-      <c r="K50" s="3" t="n"/>
+      <c r="A50" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>TPU 95A (kg)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Füße</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F50" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="3">
+        <f>E50+F50</f>
+        <v/>
+      </c>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="9">
+        <f>IF(H50="","",G50*H50)</f>
+        <v/>
+      </c>
+      <c r="J50" s="10" t="n"/>
+      <c r="K50" s="10" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="n"/>
-      <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I51" s="11">
-        <f>SUM(I2:I49)</f>
-        <v/>
-      </c>
-      <c r="J51" s="3" t="n"/>
-      <c r="K51" s="3" t="n"/>
+      <c r="A51" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>PLA orange (kg)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F51" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="3">
+        <f>E51+F51</f>
+        <v/>
+      </c>
+      <c r="H51" s="8" t="n"/>
+      <c r="I51" s="9">
+        <f>IF(H51="","",G51*H51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="10" t="n"/>
+      <c r="K51" s="10" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -2500,21 +2541,54 @@
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I52" s="3">
-        <f>COUNT(H2:H49)&amp;" von 48"</f>
-        <v/>
-      </c>
+      <c r="H52" s="3" t="n"/>
+      <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="3" t="n"/>
     </row>
+    <row r="53">
+      <c r="A53" s="3" t="n"/>
+      <c r="B53" s="3" t="n"/>
+      <c r="C53" s="3" t="n"/>
+      <c r="D53" s="3" t="n"/>
+      <c r="E53" s="3" t="n"/>
+      <c r="F53" s="3" t="n"/>
+      <c r="G53" s="3" t="n"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I53" s="11">
+        <f>SUM(I2:I51)</f>
+        <v/>
+      </c>
+      <c r="J53" s="3" t="n"/>
+      <c r="K53" s="3" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n"/>
+      <c r="B54" s="3" t="n"/>
+      <c r="C54" s="3" t="n"/>
+      <c r="D54" s="3" t="n"/>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="n"/>
+      <c r="G54" s="3" t="n"/>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I54" s="3">
+        <f>COUNT(H2:H51)&amp;" von 50"</f>
+        <v/>
+      </c>
+      <c r="J54" s="3" t="n"/>
+      <c r="K54" s="3" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2529,7 +2603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3221,7 +3295,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Stereo-Makro V1.3 / Stereo_Mount</t>
+          <t>Stereo-Makro V1.4 / Stereo_Mount</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -3261,63 +3335,116 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Rückenpanzer vorn</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>slarc_cover_v1.py / Cover_Front</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G16" s="12">
+        <f>E16*F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I16" s="13">
+        <f>D16*G16*H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>100 % (Gitter, 4 Wände)</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Grundfläche aufs Bett, ohne Stützen</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Summe nach Material</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Rückenpanzer hinten</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>slarc_cover_v1.py / Cover_Rear</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G17" s="12">
+        <f>E17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I17" s="13">
+        <f>D17*G17*H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>100 % (Gitter, 4 Wände)</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Grundfläche aufs Bett, ohne Stützen</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>PETG</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n"/>
       <c r="C18" s="3" t="n"/>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I18" s="13">
-        <f>SUMIFS(I2:I15,C2:C15,A18)</f>
-        <v/>
-      </c>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>TPU 95A</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Summe nach Material</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
@@ -3326,22 +3453,15 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I19" s="13">
-        <f>SUMIFS(I2:I15,C2:C15,A19)</f>
-        <v/>
-      </c>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>PLA</t>
+          <t>PETG</t>
         </is>
       </c>
       <c r="B20" s="3" t="n"/>
@@ -3356,16 +3476,16 @@
         </is>
       </c>
       <c r="I20" s="13">
-        <f>SUMIFS(I2:I15,C2:C15,A20)</f>
+        <f>SUMIFS(I2:I17,C2:C17,A20)</f>
         <v/>
       </c>
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Alle Druckteile</t>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>TPU 95A</t>
         </is>
       </c>
       <c r="B21" s="3" t="n"/>
@@ -3374,13 +3494,61 @@
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="14">
-        <f>SUM(I18:I20)</f>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I21" s="13">
+        <f>SUMIFS(I2:I17,C2:C17,A21)</f>
         <v/>
       </c>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>PLA</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I22" s="13">
+        <f>SUMIFS(I2:I17,C2:C17,A22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Alle Druckteile</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="14">
+        <f>SUM(I20:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="3" t="n"/>
+      <c r="K23" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3426,7 +3594,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Druckteile!I21</f>
+        <f>Druckteile!I23</f>
         <v/>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Cover V1.1: lighter back shell (~170 g instead of ~270 g)
- wall 3.0 -> 2.4 mm, honeycomb 9 mm / rib 2.4 mm, diamond windows in
  the side walls, narrower intermediate frames (3 mm, 5 mm flange),
  hollow posts, crest 3 mm wide
- 6 posts instead of 8 (the split frame carries at x = -40); roof skin
  kept closed around each post
- one intermediate frame removed (x = 40)
- BOM: volumes, 6x M3x50 + 6 inserts, 2x M3x45 remain at x = -40

Checked in FreeCAD: both parts single valid solids, no overlaps with
electronics/servos, base fully on plate, no overhang > 55 deg except
small hole tops.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1776,11 +1776,11 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Säulen obere/untere Platte, von unten in den Gewindeeinsatz des Panzers (ohne Panzer: M3x45 + Mutter)</t>
+          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F31" s="7" t="n">
         <v>1</v>
@@ -1813,11 +1813,11 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>unten in den 8 Panzersäulen</t>
+          <t>unten in den 6 Panzersäulen</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F32" s="7" t="n">
         <v>2</v>
@@ -1845,16 +1845,16 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12 + Mutter</t>
+          <t>Zylinderschraube M3x45</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" s="7" t="n">
         <v>1</v>
@@ -1882,19 +1882,19 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G34" s="3">
         <f>E34+F34</f>
@@ -1919,19 +1919,19 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Säulen + Stoß + Relais</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G35" s="3">
         <f>E35+F35</f>
@@ -1956,19 +1956,19 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Säulen + Stoß + Relais</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F36" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="F36" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G36" s="3">
         <f>E36+F36</f>
@@ -1993,19 +1993,19 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Zylinderschraube M3x14</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4)</t>
+          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3">
         <f>E37+F37</f>
@@ -2030,16 +2030,16 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4)</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F38" s="7" t="n">
         <v>2</v>
@@ -2067,19 +2067,19 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Zylinderschraube M2x6</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F39" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F39" s="7" t="n">
-        <v>1</v>
       </c>
       <c r="G39" s="3">
         <f>E39+F39</f>
@@ -2104,19 +2104,19 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+          <t>Zylinderschraube M2x25 + Mutter</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Pi 5 (M2 geht mit Scheiben)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="3">
         <f>E40+F40</f>
@@ -2141,12 +2141,12 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+          <t>Pi 5 (M2 geht mit Scheiben)</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
@@ -2178,19 +2178,19 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>für die Distanzbolzen, je 2</t>
+          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G42" s="3">
         <f>E42+F42</f>
@@ -2215,15 +2215,19 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr"/>
+          <t>Zylinderschraube M2,5x5</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>für die Distanzbolzen, je 2</t>
+        </is>
+      </c>
       <c r="E43" s="7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G43" s="3">
         <f>E43+F43</f>
@@ -2248,14 +2252,10 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr"/>
       <c r="E44" s="7" t="n">
         <v>1</v>
       </c>
@@ -2280,21 +2280,21 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F45" s="7" t="n">
         <v>0</v>
@@ -2322,16 +2322,16 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F46" s="7" t="n">
         <v>0</v>
@@ -2359,12 +2359,12 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
@@ -2396,12 +2396,12 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
@@ -2428,21 +2428,21 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" s="7" t="n">
         <v>0</v>
@@ -2470,16 +2470,16 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="F50" s="7" t="n">
         <v>0</v>
@@ -2507,16 +2507,16 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>PLA orange (kg)</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="F51" s="7" t="n">
         <v>0</v>
@@ -2534,17 +2534,41 @@
       <c r="K51" s="10" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="n"/>
-      <c r="B52" s="3" t="n"/>
-      <c r="C52" s="3" t="n"/>
-      <c r="D52" s="3" t="n"/>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="n"/>
-      <c r="I52" s="3" t="n"/>
-      <c r="J52" s="3" t="n"/>
-      <c r="K52" s="3" t="n"/>
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>PLA orange (kg)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F52" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="3">
+        <f>E52+F52</f>
+        <v/>
+      </c>
+      <c r="H52" s="8" t="n"/>
+      <c r="I52" s="9">
+        <f>IF(H52="","",G52*H52)</f>
+        <v/>
+      </c>
+      <c r="J52" s="10" t="n"/>
+      <c r="K52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -2554,15 +2578,8 @@
       <c r="E53" s="3" t="n"/>
       <c r="F53" s="3" t="n"/>
       <c r="G53" s="3" t="n"/>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I53" s="11">
-        <f>SUM(I2:I51)</f>
-        <v/>
-      </c>
+      <c r="H53" s="3" t="n"/>
+      <c r="I53" s="3" t="n"/>
       <c r="J53" s="3" t="n"/>
       <c r="K53" s="3" t="n"/>
     </row>
@@ -2574,21 +2591,41 @@
       <c r="E54" s="3" t="n"/>
       <c r="F54" s="3" t="n"/>
       <c r="G54" s="3" t="n"/>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I54" s="3">
-        <f>COUNT(H2:H51)&amp;" von 50"</f>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I54" s="11">
+        <f>SUM(I2:I52)</f>
         <v/>
       </c>
       <c r="J54" s="3" t="n"/>
       <c r="K54" s="3" t="n"/>
     </row>
+    <row r="55">
+      <c r="A55" s="3" t="n"/>
+      <c r="B55" s="3" t="n"/>
+      <c r="C55" s="3" t="n"/>
+      <c r="D55" s="3" t="n"/>
+      <c r="E55" s="3" t="n"/>
+      <c r="F55" s="3" t="n"/>
+      <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I55" s="3">
+        <f>COUNT(H2:H52)&amp;" von 51"</f>
+        <v/>
+      </c>
+      <c r="J55" s="3" t="n"/>
+      <c r="K55" s="3" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3354,7 +3391,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>122.5</v>
+        <v>79.8</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>1.27</v>
@@ -3364,7 +3401,7 @@
         <v/>
       </c>
       <c r="H16" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I16" s="13">
         <f>D16*G16*H16</f>
@@ -3401,7 +3438,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>96.5</v>
+        <v>66.3</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>1.27</v>
@@ -3411,7 +3448,7 @@
         <v/>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I17" s="13">
         <f>D17*G17*H17</f>

</xml_diff>

<commit_message>
Battery latch: no half-shells in the battery exit path
The 12 mm half-shells stood behind the battery and blocked it from being
pulled out. Now nothing stays on the bottom plate once the pins are pulled:
- pins are guided at both ends: bottom plate (bayonet slot + detent notch
  in the plate top) and a guide bore in the top plate (chamfered below)
- rear end of the battery pocket is a 4 mm ramp instead of a 2 mm step
- FreeCAD check: battery pulled out 170 mm with pins removed, no contact
  with bottom plate, top plate or connector holder
- BOM volumes updated (bottom rear, top rear, pin)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -3185,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>88.7</v>
+        <v>88.19</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>1.27</v>
@@ -3279,7 +3279,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>88.73</v>
+        <v>87.11</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>1.27</v>
@@ -3420,7 +3420,7 @@
         <v>2</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>3.15</v>
+        <v>3.63</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>1.27</v>

</xml_diff>

<commit_message>
Battery latch: one centered pin between the battery cable exits
Balancer and main lead leave the battery end face near the sides; two pins
at y +-16 could collide with them. One pin at y 0 sits in the gap.
BOM: latch pin x1, foam pad x1, rear plate volumes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 2 Stücke 20x20 mit Ø9-Loch unter die Köpfe der Akku-Riegel</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
@@ -3185,7 +3185,7 @@
         <v>1</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>88.19</v>
+        <v>88.45</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>1.27</v>
@@ -3279,7 +3279,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>87.11</v>
+        <v>87.37</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>1.27</v>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>3.63</v>

</xml_diff>

<commit_message>
Stereo mount V1.5: rounded corners
- Upper frame corners R6 (front view), inner board corner stays square,
  min. wall 1.76 mm
- Ear ends fully rounded (R2), fillet R2.5 between frame and ear
  (M3 screw head stays clear)
- Same geometry in the copy in the baseplate macro (checked: identical)
- STL, BOM (volume, print hint: brim, fan from layer 4), README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Konstruktion: Bein V9.1 (Femur 150, Tibia 175, Knick 38,6°), Baseplates V2.7 (DC-DC, Modulplätze, Steckerhalter, Akku-Riegel), Kamerahalter V1.4, Panzer V1.1</t>
+          <t>Konstruktion: Bein V9.1 (Femur 150, Tibia 175, Knick 38,6°), Baseplates V2.7 (DC-DC, Modulplätze, Steckerhalter, Akku-Riegel), Kamerahalter V1.5, Panzer V1.1</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Stereo-Makro V1.4 / Stereo_Mount</t>
+          <t>Stereo-Makro V1.5 / Stereo_Mount</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -3326,7 +3326,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>31</v>
+        <v>30.7</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>1.27</v>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Frontfläche aufs Bett</t>
+          <t>Frontfläche aufs Bett, Brim 6–8 mm, Lüfter erst ab Schicht 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wiring plan and perfboard layouts
- Documentation/Wiring: block diagram, current budget and wire gauges,
  wire list, ESP32/Pi pin assignment, power-on sequence, commissioning
- perfboard layouts (SVG, generated by gen_wiring_svg.py): A leg
  distributor (6x), B hub with MCP23017 + data star, C power distributor,
  D relay adapter (diodes for the ESP32, BC547 for the Pi hold)
- BOM: parts for the boards (470 uF, 100 nF, BC547, 4k7, DIP-28 socket,
  headers, AWG24/AWG14, bus-bar copper), MCP23017 as DIP-28
- README: power line and repo structure

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -908,12 +908,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>IO-Expander MCP23017 (Breakout)</t>
+          <t>IO-Expander MCP23017-E/SP (DIP-28)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>I2C, 6 Fußkontakte + Status-LEDs an Bank B; INTA -&gt; GPIO34/35</t>
+          <t>auf Hub-Platine B, Adresse 0x20; 6 Fußkontakte an GPA0–5, INTA -&gt; IO34; Bank B frei für Status-LEDs</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Daten an IO4 (3-pol. Servoanschluss Treiberboard), 5 V vom DC-DC</t>
+          <t>Daten an IO4; 5 V vom Treiber (bis ~10 LEDs) oder vom DC-DC</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>oder kleineres 2–4-Kanal-Modul</t>
+          <t>K1 schaltet 12 V zum DC-DC (Pi), K2/K3 Servos links/rechts; 5-V-Spule, Eingänge aktiv-low, Kontakte 10 A</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
@@ -1431,14 +1431,14 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Stromschienen je Seite</t>
+          <t>vorhanden; Speisung je Bein (Paar), Relais, DC-DC, Pi-5V (je Pol 2 Adern)</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="3">
         <f>E22+F22</f>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Verteilerplatine je Bein (Lochraster, XH2.54)</t>
+          <t>Bein-Platine A (Lochraster ½ 3×7 cm)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Eigenbau</t>
+          <t>Eigenbau, Layout Documentation/Wiring</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
@@ -1538,11 +1538,11 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Abschaltschaltung Pi</t>
+          <t>Relais-Adapter (Platine D): ESP32 -&gt; K1, K2, K3</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" s="7" t="n">
         <v>2</v>
@@ -1602,24 +1602,24 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
+          <t>je Bein-Platine, + an 12 V</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G27" s="3">
         <f>E27+F27</f>
@@ -1639,24 +1639,24 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x6</t>
+          <t>Keramikkondensator 100 nF</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
+          <t>Abblockung MCP23017 (Hub)</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G28" s="3">
         <f>E28+F28</f>
@@ -1676,24 +1676,24 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
+          <t>Transistor BC547 (NPN)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
+          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="3">
         <f>E29+F29</f>
@@ -1713,24 +1713,24 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x50</t>
+          <t>Widerstand 4,7 kΩ</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
+          <t>Basiswiderstand BC547</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" s="3">
         <f>E30+F30</f>
@@ -1750,24 +1750,24 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
+          <t>IC-Fassung DIP-28</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>unten in den 6 Panzersäulen</t>
+          <t>für MCP23017 (Hub)</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="3">
         <f>E31+F31</f>
@@ -1787,24 +1787,24 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
+          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F32" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="3">
         <f>E32+F32</f>
@@ -1824,24 +1824,24 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12 + Mutter</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>Relais-Adapter auf Modul-Eingangsleiste</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33" s="3">
         <f>E33+F33</f>
@@ -1861,24 +1861,24 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Lochrasterplatinen AZ-Delivery</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G34" s="3">
         <f>E34+F34</f>
@@ -1898,24 +1898,24 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Säulen + Stoß + Relais</t>
+          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G35" s="3">
         <f>E35+F35</f>
@@ -1935,21 +1935,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Litze AWG14 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F36" s="7" t="n">
         <v>0</v>
@@ -1972,24 +1972,24 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4) + Steckerhalter Akku (2)</t>
+          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>8</v>
+        <v>0.5</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3">
         <f>E37+F37</f>
@@ -2009,24 +2009,24 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>Schienen Bein-Platinen und Hub</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="3">
         <f>E38+F38</f>
@@ -2046,24 +2046,24 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Servokabel 5264 3-pol.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G39" s="3">
         <f>E39+F39</f>
@@ -2088,19 +2088,19 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Pi 5 (M2 geht mit Scheiben)</t>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G40" s="3">
         <f>E40+F40</f>
@@ -2125,19 +2125,19 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+          <t>Zylinderschraube M3x6</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>4</v>
+        <v>72</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G41" s="3">
         <f>E41+F41</f>
@@ -2162,19 +2162,19 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>für die Distanzbolzen, je 2</t>
+          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G42" s="3">
         <f>E42+F42</f>
@@ -2199,15 +2199,19 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n"/>
+          <t>Zylinderschraube M3x50</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
+        </is>
+      </c>
       <c r="E43" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="3">
         <f>E43+F43</f>
@@ -2232,19 +2236,19 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
+          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
+          <t>unten in den 6 Panzersäulen</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G44" s="3">
         <f>E44+F44</f>
@@ -2264,24 +2268,24 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Zylinderschraube M3x45</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" s="3">
         <f>E45+F45</f>
@@ -2301,24 +2305,24 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" s="3">
         <f>E46+F46</f>
@@ -2338,24 +2342,24 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G47" s="3">
         <f>E47+F47</f>
@@ -2375,24 +2379,24 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Säulen + Stoß + Relais</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G48" s="3">
         <f>E48+F48</f>
@@ -2412,21 +2416,21 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>Zylinderschraube M3x14</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F49" s="7" t="n">
         <v>0</v>
@@ -2449,24 +2453,24 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4) + Steckerhalter Akku (2)</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F50" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F50" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G50" s="3">
         <f>E50+F50</f>
@@ -2486,24 +2490,24 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>Zylinderschraube M2x6</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>0.25</v>
+        <v>8</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G51" s="3">
         <f>E51+F51</f>
@@ -2523,24 +2527,24 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>PLA orange (kg)</t>
+          <t>Zylinderschraube M2x25 + Mutter</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52" s="3">
         <f>E52+F52</f>
@@ -2555,61 +2559,538 @@
       <c r="K52" s="10" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="n"/>
-      <c r="B53" s="3" t="n"/>
-      <c r="C53" s="3" t="n"/>
-      <c r="D53" s="3" t="n"/>
-      <c r="E53" s="3" t="n"/>
-      <c r="F53" s="3" t="n"/>
-      <c r="G53" s="3" t="n"/>
-      <c r="H53" s="3" t="n"/>
-      <c r="I53" s="3" t="n"/>
-      <c r="J53" s="3" t="n"/>
-      <c r="K53" s="3" t="n"/>
+      <c r="A53" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Verbindung</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Pi 5 (M2 geht mit Scheiben)</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F53" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="3">
+        <f>E53+F53</f>
+        <v/>
+      </c>
+      <c r="H53" s="8" t="n"/>
+      <c r="I53" s="9">
+        <f>IF(H53="","",G53*H53)</f>
+        <v/>
+      </c>
+      <c r="J53" s="10" t="n"/>
+      <c r="K53" s="10" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="n"/>
-      <c r="B54" s="3" t="n"/>
-      <c r="C54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="A54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Verbindung</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F54" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="3">
+        <f>E54+F54</f>
+        <v/>
+      </c>
+      <c r="H54" s="8" t="n"/>
+      <c r="I54" s="9">
+        <f>IF(H54="","",G54*H54)</f>
+        <v/>
+      </c>
+      <c r="J54" s="10" t="n"/>
+      <c r="K54" s="10" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Verbindung</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M2,5x5</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>für die Distanzbolzen, je 2</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" s="3">
+        <f>E55+F55</f>
+        <v/>
+      </c>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="9">
+        <f>IF(H55="","",G55*H55)</f>
+        <v/>
+      </c>
+      <c r="J55" s="10" t="n"/>
+      <c r="K55" s="10" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Verbindung</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n"/>
+      <c r="E56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="3">
+        <f>E56+F56</f>
+        <v/>
+      </c>
+      <c r="H56" s="8" t="n"/>
+      <c r="I56" s="9">
+        <f>IF(H56="","",G56*H56)</f>
+        <v/>
+      </c>
+      <c r="J56" s="10" t="n"/>
+      <c r="K56" s="10" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Verbindung</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Federstahldraht 1,2 mm (m)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="3">
+        <f>E57+F57</f>
+        <v/>
+      </c>
+      <c r="H57" s="8" t="n"/>
+      <c r="I57" s="9">
+        <f>IF(H57="","",G57*H57)</f>
+        <v/>
+      </c>
+      <c r="J57" s="10" t="n"/>
+      <c r="K57" s="10" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Kleinteile</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Kabelbinder 2,5 mm</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Kabelösen Femur/Tibia</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="F58" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="3">
+        <f>E58+F58</f>
+        <v/>
+      </c>
+      <c r="H58" s="8" t="n"/>
+      <c r="I58" s="9">
+        <f>IF(H58="","",G58*H58)</f>
+        <v/>
+      </c>
+      <c r="J58" s="10" t="n"/>
+      <c r="K58" s="10" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Kleinteile</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Klettband 20 mm (m)</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="3">
+        <f>E59+F59</f>
+        <v/>
+      </c>
+      <c r="H59" s="8" t="n"/>
+      <c r="I59" s="9">
+        <f>IF(H59="","",G59*H59)</f>
+        <v/>
+      </c>
+      <c r="J59" s="10" t="n"/>
+      <c r="K59" s="10" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Kleinteile</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="3">
+        <f>E60+F60</f>
+        <v/>
+      </c>
+      <c r="H60" s="8" t="n"/>
+      <c r="I60" s="9">
+        <f>IF(H60="","",G60*H60)</f>
+        <v/>
+      </c>
+      <c r="J60" s="10" t="n"/>
+      <c r="K60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Kleinteile</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Doppelseitiges Klebeband</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Trigger-Platine</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="3">
+        <f>E61+F61</f>
+        <v/>
+      </c>
+      <c r="H61" s="8" t="n"/>
+      <c r="I61" s="9">
+        <f>IF(H61="","",G61*H61)</f>
+        <v/>
+      </c>
+      <c r="J61" s="10" t="n"/>
+      <c r="K61" s="10" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Kleinteile</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="3">
+        <f>E62+F62</f>
+        <v/>
+      </c>
+      <c r="H62" s="8" t="n"/>
+      <c r="I62" s="9">
+        <f>IF(H62="","",G62*H62)</f>
+        <v/>
+      </c>
+      <c r="J62" s="10" t="n"/>
+      <c r="K62" s="10" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>PETG schwarz (kg)</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="3">
+        <f>E63+F63</f>
+        <v/>
+      </c>
+      <c r="H63" s="8" t="n"/>
+      <c r="I63" s="9">
+        <f>IF(H63="","",G63*H63)</f>
+        <v/>
+      </c>
+      <c r="J63" s="10" t="n"/>
+      <c r="K63" s="10" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>TPU 95A (kg)</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Füße</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="3">
+        <f>E64+F64</f>
+        <v/>
+      </c>
+      <c r="H64" s="8" t="n"/>
+      <c r="I64" s="9">
+        <f>IF(H64="","",G64*H64)</f>
+        <v/>
+      </c>
+      <c r="J64" s="10" t="n"/>
+      <c r="K64" s="10" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>PLA orange (kg)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F65" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="3">
+        <f>E65+F65</f>
+        <v/>
+      </c>
+      <c r="H65" s="8" t="n"/>
+      <c r="I65" s="9">
+        <f>IF(H65="","",G65*H65)</f>
+        <v/>
+      </c>
+      <c r="J65" s="10" t="n"/>
+      <c r="K65" s="10" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n"/>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="n"/>
+      <c r="I66" s="3" t="n"/>
+      <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n"/>
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+      <c r="G67" s="3" t="n"/>
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="I54" s="11">
-        <f>SUM(I2:I52)</f>
-        <v/>
-      </c>
-      <c r="J54" s="3" t="n"/>
-      <c r="K54" s="3" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="n"/>
-      <c r="B55" s="3" t="n"/>
-      <c r="C55" s="3" t="n"/>
-      <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="I67" s="11">
+        <f>SUM(I2:I65)</f>
+        <v/>
+      </c>
+      <c r="J67" s="3" t="n"/>
+      <c r="K67" s="3" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n"/>
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="inlineStr">
         <is>
           <t>Preise erfasst</t>
         </is>
       </c>
-      <c r="I55" s="3">
-        <f>COUNT(H2:H52)&amp;" von 51"</f>
-        <v/>
-      </c>
-      <c r="J55" s="3" t="n"/>
-      <c r="K55" s="3" t="n"/>
+      <c r="I68" s="3">
+        <f>COUNT(H2:H65)&amp;" von 64"</f>
+        <v/>
+      </c>
+      <c r="J68" s="3" t="n"/>
+      <c r="K68" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Wiring: one relay per leg, MCP23017 module, relay module without diodes
- K2..K7 switch one leg each (max 8.1 A < 10 A contact rating);
  one relay per side (~15 A peak) would be overloaded
- relay module with JD-VCC jumper removed: opto side 3.3 V, coils 5 V,
  inputs driven directly by 3.3 V logic; IO16 open-drain, Pi via BC547
- hub board for the MCP23017-E breakout (20-pin side header), I2C/INT
  straight to the module's top header
- power board reduced to two bus bars (12 V, GND)
- BOM: MCP23017 module, relay spec, 1N4148 and DIP socket removed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -908,12 +908,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>IO-Expander MCP23017-E/SP (DIP-28)</t>
+          <t>IO-Expander MCP23017-E (Modul/Breakout)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>auf Hub-Platine B, Adresse 0x20; 6 Fußkontakte an GPA0–5, INTA -&gt; IO34; Bank B frei für Status-LEDs</t>
+          <t>auf Hub-Platine B (seitliche Stiftleiste); Adresse 0x20 (A0–A2 auf GND); Füße an PA0–5, ITA -&gt; IO34; ~7,30 €</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>K1 schaltet 12 V zum DC-DC (Pi), K2/K3 Servos links/rechts; 5-V-Spule, Eingänge aktiv-low, Kontakte 10 A</t>
+          <t>8× SRD-05VDC-SL-C (10 A): K1 12 V -&gt; DC-DC (Pi), K2–K7 je ein Bein, K8 frei; Jumper JD-VCC ziehen (VCC 3,3 V, JD-VCC 5 V)</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>vorhanden; Speisung je Bein (Paar), Relais, DC-DC, Pi-5V (je Pol 2 Adern)</t>
+          <t>vorhanden; je Bein 12 V (von Kx NO) + GND, Relais-COM, DC-DC, Pi-5V (je Pol 2 Adern)</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
@@ -1533,16 +1533,16 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Diode 1N4148</t>
+          <t>Dupont-Kabel (Trigger/Strobe)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter (Platine D): ESP32 -&gt; K1, K2, K3</t>
+          <t>Kameras &lt;-&gt; Trigger-Platine</t>
         </is>
       </c>
       <c r="E25" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F25" s="7" t="n">
         <v>2</v>
@@ -1570,16 +1570,16 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Dupont-Kabel (Trigger/Strobe)</t>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Kameras &lt;-&gt; Trigger-Platine</t>
+          <t>je Bein-Platine, + an 12 V</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F26" s="7" t="n">
         <v>2</v>
@@ -1607,19 +1607,19 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
+          <t>Keramikkondensator 100 nF</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>je Bein-Platine, + an 12 V</t>
+          <t>Abblockung MCP23017 (Hub)</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G27" s="3">
         <f>E27+F27</f>
@@ -1644,19 +1644,19 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Keramikkondensator 100 nF</t>
+          <t>Transistor BC547 (NPN)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Abblockung MCP23017 (Hub)</t>
+          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G28" s="3">
         <f>E28+F28</f>
@@ -1681,19 +1681,19 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Transistor BC547 (NPN)</t>
+          <t>Widerstand 4,7 kΩ</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
+          <t>Basiswiderstand BC547</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="3">
         <f>E29+F29</f>
@@ -1718,19 +1718,19 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Widerstand 4,7 kΩ</t>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Basiswiderstand BC547</t>
+          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3">
         <f>E30+F30</f>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>IC-Fassung DIP-28</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>für MCP23017 (Hub)</t>
+          <t>Relais-Adapter auf Modul-Eingangsleiste (optional 20-pol. für das MCP-Modul)</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -1792,16 +1792,16 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
+          <t>Lochrasterplatinen AZ-Delivery</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
+          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" s="7" t="n">
         <v>0</v>
@@ -1829,16 +1829,16 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Buchsenleiste 2,54 mm, 10-pol.</t>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter auf Modul-Eingangsleiste</t>
+          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F33" s="7" t="n">
         <v>0</v>
@@ -1861,17 +1861,17 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Lochrasterplatinen AZ-Delivery</t>
+          <t>Litze AWG14 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
+          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
@@ -1903,16 +1903,16 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
+          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>10</v>
+        <v>0.5</v>
       </c>
       <c r="F35" s="7" t="n">
         <v>0</v>
@@ -1935,21 +1935,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Litze AWG14 rot/schwarz (m)</t>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
+          <t>Schienen Bein-Platinen und Hub</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" s="7" t="n">
         <v>0</v>
@@ -1977,19 +1977,19 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Kupferdraht 1,5 mm² massiv (m)</t>
+          <t>Servokabel 5264 3-pol.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
+          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G37" s="3">
         <f>E37+F37</f>
@@ -2009,24 +2009,24 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
+          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Schienen Bein-Platinen und Hub</t>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G38" s="3">
         <f>E38+F38</f>
@@ -2046,24 +2046,24 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Servokabel 5264 3-pol.</t>
+          <t>Zylinderschraube M3x6</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
+          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G39" s="3">
         <f>E39+F39</f>
@@ -2088,19 +2088,19 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
+          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
+          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G40" s="3">
         <f>E40+F40</f>
@@ -2125,19 +2125,19 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x6</t>
+          <t>Zylinderschraube M3x50</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
+          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>72</v>
+        <v>6</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G41" s="3">
         <f>E41+F41</f>
@@ -2162,19 +2162,19 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
+          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
+          <t>unten in den 6 Panzersäulen</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G42" s="3">
         <f>E42+F42</f>
@@ -2199,16 +2199,16 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x50</t>
+          <t>Zylinderschraube M3x45</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
+          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F43" s="7" t="n">
         <v>1</v>
@@ -2236,19 +2236,19 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>unten in den 6 Panzersäulen</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G44" s="3">
         <f>E44+F44</f>
@@ -2273,19 +2273,19 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F45" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F45" s="7" t="n">
-        <v>1</v>
       </c>
       <c r="G45" s="3">
         <f>E45+F45</f>
@@ -2310,19 +2310,19 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12 + Mutter</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>Säulen + Stoß + Relais</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G46" s="3">
         <f>E46+F46</f>
@@ -2347,19 +2347,19 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Zylinderschraube M3x14</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G47" s="3">
         <f>E47+F47</f>
@@ -2384,19 +2384,19 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Säulen + Stoß + Relais</t>
+          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4) + Steckerhalter Akku (2)</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G48" s="3">
         <f>E48+F48</f>
@@ -2421,19 +2421,19 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Zylinderschraube M2x6</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G49" s="3">
         <f>E49+F49</f>
@@ -2458,19 +2458,19 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Zylinderschraube M2x25 + Mutter</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4) + Steckerhalter Akku (2)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" s="3">
         <f>E50+F50</f>
@@ -2495,19 +2495,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>Pi 5 (M2 geht mit Scheiben)</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G51" s="3">
         <f>E51+F51</f>
@@ -2532,19 +2532,19 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G52" s="3">
         <f>E52+F52</f>
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+          <t>Zylinderschraube M2,5x5</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Pi 5 (M2 geht mit Scheiben)</t>
+          <t>für die Distanzbolzen, je 2</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G53" s="3">
         <f>E53+F53</f>
@@ -2606,16 +2606,12 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n"/>
       <c r="E54" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F54" s="7" t="n">
         <v>0</v>
@@ -2643,19 +2639,19 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>für die Distanzbolzen, je 2</t>
+          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G55" s="3">
         <f>E55+F55</f>
@@ -2675,17 +2671,21 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="n"/>
+          <t>Kabelbinder 2,5 mm</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Kabelösen Femur/Tibia</t>
+        </is>
+      </c>
       <c r="E56" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F56" s="7" t="n">
         <v>0</v>
@@ -2708,17 +2708,17 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
@@ -2750,16 +2750,16 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F58" s="7" t="n">
         <v>0</v>
@@ -2787,12 +2787,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -2824,12 +2824,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -2856,21 +2856,21 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="7" t="n">
         <v>0</v>
@@ -2893,21 +2893,21 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F62" s="7" t="n">
         <v>0</v>
@@ -2935,16 +2935,16 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>PLA orange (kg)</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="F63" s="7" t="n">
         <v>0</v>
@@ -2962,78 +2962,37 @@
       <c r="K63" s="10" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Filament</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>TPU 95A (kg)</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Füße</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F64" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" s="3">
-        <f>E64+F64</f>
-        <v/>
-      </c>
-      <c r="H64" s="8" t="n"/>
-      <c r="I64" s="9">
-        <f>IF(H64="","",G64*H64)</f>
-        <v/>
-      </c>
-      <c r="J64" s="10" t="n"/>
-      <c r="K64" s="10" t="n"/>
+      <c r="A64" s="3" t="n"/>
+      <c r="B64" s="3" t="n"/>
+      <c r="C64" s="3" t="n"/>
+      <c r="D64" s="3" t="n"/>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
+      <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
+      <c r="I64" s="3" t="n"/>
+      <c r="J64" s="3" t="n"/>
+      <c r="K64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>Filament</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>PLA orange (kg)</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>Zierleisten</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F65" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="3">
-        <f>E65+F65</f>
-        <v/>
-      </c>
-      <c r="H65" s="8" t="n"/>
-      <c r="I65" s="9">
-        <f>IF(H65="","",G65*H65)</f>
-        <v/>
-      </c>
-      <c r="J65" s="10" t="n"/>
-      <c r="K65" s="10" t="n"/>
+      <c r="A65" s="3" t="n"/>
+      <c r="B65" s="3" t="n"/>
+      <c r="C65" s="3" t="n"/>
+      <c r="D65" s="3" t="n"/>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="3" t="n"/>
+      <c r="G65" s="3" t="n"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I65" s="11">
+        <f>SUM(I2:I63)</f>
+        <v/>
+      </c>
+      <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -3043,54 +3002,21 @@
       <c r="E66" s="3" t="n"/>
       <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="n"/>
-      <c r="I66" s="3" t="n"/>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I66" s="3">
+        <f>COUNT(H2:H63)&amp;" von 62"</f>
+        <v/>
+      </c>
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="3" t="n"/>
     </row>
-    <row r="67">
-      <c r="A67" s="3" t="n"/>
-      <c r="B67" s="3" t="n"/>
-      <c r="C67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
-      <c r="F67" s="3" t="n"/>
-      <c r="G67" s="3" t="n"/>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I67" s="11">
-        <f>SUM(I2:I65)</f>
-        <v/>
-      </c>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="3" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="n"/>
-      <c r="B68" s="3" t="n"/>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
-      <c r="G68" s="3" t="n"/>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I68" s="3">
-        <f>COUNT(H2:H65)&amp;" von 64"</f>
-        <v/>
-      </c>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="3" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Baseplate V2.8: places and mounts for the perfboards
- leg boards A (half 3x7) between the plates on M2 bosses of the bottom
  plate: FR/FL x 183, MR/ML x 0, RR/RL x -100 (outside the battery path)
- hub B (5x7, holes 66x46) on a printed carrier at the MCP module spot,
  module side outward where the shell is low
- power board C on a printed bridge over the BMS, resting on two sleeves
  slipped over the columns (60, +-45)
- relay adapter D in front of the relay module (angled female header)
- placeholders checked against servos, battery path, relay, BMS, holder,
  columns and back shell; STLs for carrier, bridge, sleeve; BOM updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Buchsenleiste 2,54 mm, 10-pol.</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter auf Modul-Eingangsleiste (optional 20-pol. für das MCP-Modul)</t>
+          <t>Relais-Adapter auf die Eingangsstifte des Relaismoduls (nur ~16 mm Höhe frei)</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
@@ -2389,11 +2389,11 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Modulträger MCP/MUX (4) + Steckerhalter Akku (2)</t>
+          <t>DC-DC-Laschen (2) + Hub-Träger auf Modulplatz MCP (2) + Steckerhalter Akku (2)</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F48" s="7" t="n">
         <v>2</v>
@@ -2458,19 +2458,19 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Zylinderschraube M2x5</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>Lochraster-Platinen: 6× Bein (je 2), Hub (4), Power-Verteiler (2), direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G50" s="3">
         <f>E50+F50</f>
@@ -2495,19 +2495,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+          <t>Zylinderschraube M2x25 + Mutter</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Pi 5 (M2 geht mit Scheiben)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G51" s="3">
         <f>E51+F51</f>
@@ -2532,12 +2532,12 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+          <t>Pi 5 (M2 geht mit Scheiben)</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>für die Distanzbolzen, je 2</t>
+          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G53" s="3">
         <f>E53+F53</f>
@@ -2606,15 +2606,19 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="n"/>
+          <t>Zylinderschraube M2,5x5</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>für die Distanzbolzen, je 2</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G54" s="3">
         <f>E54+F54</f>
@@ -2639,14 +2643,10 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n"/>
       <c r="E55" s="7" t="n">
         <v>1</v>
       </c>
@@ -2671,21 +2671,21 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
         </is>
       </c>
       <c r="E56" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F56" s="7" t="n">
         <v>0</v>
@@ -2713,16 +2713,16 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F57" s="7" t="n">
         <v>0</v>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
@@ -2787,12 +2787,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -2824,12 +2824,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -2856,21 +2856,21 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" s="7" t="n">
         <v>0</v>
@@ -2898,16 +2898,16 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="F62" s="7" t="n">
         <v>0</v>
@@ -2935,16 +2935,16 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>PLA orange (kg)</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="F63" s="7" t="n">
         <v>0</v>
@@ -2962,17 +2962,41 @@
       <c r="K63" s="10" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n"/>
-      <c r="B64" s="3" t="n"/>
-      <c r="C64" s="3" t="n"/>
-      <c r="D64" s="3" t="n"/>
-      <c r="E64" s="3" t="n"/>
-      <c r="F64" s="3" t="n"/>
-      <c r="G64" s="3" t="n"/>
-      <c r="H64" s="3" t="n"/>
-      <c r="I64" s="3" t="n"/>
-      <c r="J64" s="3" t="n"/>
-      <c r="K64" s="3" t="n"/>
+      <c r="A64" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>PLA orange (kg)</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F64" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="3">
+        <f>E64+F64</f>
+        <v/>
+      </c>
+      <c r="H64" s="8" t="n"/>
+      <c r="I64" s="9">
+        <f>IF(H64="","",G64*H64)</f>
+        <v/>
+      </c>
+      <c r="J64" s="10" t="n"/>
+      <c r="K64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -2982,15 +3006,8 @@
       <c r="E65" s="3" t="n"/>
       <c r="F65" s="3" t="n"/>
       <c r="G65" s="3" t="n"/>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I65" s="11">
-        <f>SUM(I2:I63)</f>
-        <v/>
-      </c>
+      <c r="H65" s="3" t="n"/>
+      <c r="I65" s="3" t="n"/>
       <c r="J65" s="3" t="n"/>
       <c r="K65" s="3" t="n"/>
     </row>
@@ -3002,21 +3019,41 @@
       <c r="E66" s="3" t="n"/>
       <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I66" s="3">
-        <f>COUNT(H2:H63)&amp;" von 62"</f>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I66" s="11">
+        <f>SUM(I2:I64)</f>
         <v/>
       </c>
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="3" t="n"/>
     </row>
+    <row r="67">
+      <c r="A67" s="3" t="n"/>
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+      <c r="G67" s="3" t="n"/>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I67" s="3">
+        <f>COUNT(H2:H64)&amp;" von 63"</f>
+        <v/>
+      </c>
+      <c r="J67" s="3" t="n"/>
+      <c r="K67" s="3" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3030,7 +3067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3639,7 +3676,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>148.88</v>
+        <v>149.63</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>1.27</v>
@@ -3662,7 +3699,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Unterseite aufs Bett</t>
+          <t>Unterseite aufs Bett (V2.8: M2-Bunde für 4 Bein-Platinen)</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3723,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>87.37</v>
+        <v>87.75</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>1.27</v>
@@ -3949,87 +3986,163 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n"/>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Hub-Träger</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Baseplate-Makro V2.8 / Hub_Carrier</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G20" s="12">
+        <f>E20*F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I20" s="13">
+        <f>D20*G20*H20</f>
+        <v/>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>30 %</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Bunde nach oben, ohne Stützen</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Summe nach Material</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Power-Brücke</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Baseplate-Makro V2.8 / Power_Bridge</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G21" s="12">
+        <f>E21*F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I21" s="13">
+        <f>D21*G21*H21</f>
+        <v/>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>30 %</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Deck aufs Bett, Bunde nach oben</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>Hülse Power-Brücke</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Baseplate-Makro V2.8 / Power_Bridge_Sleeve</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
           <t>PETG</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
+      <c r="D22" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G22" s="12">
+        <f>E22*F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>1</v>
       </c>
       <c r="I22" s="13">
-        <f>SUMIFS(I2:I19,C2:C19,A22)</f>
-        <v/>
-      </c>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
+        <f>D22*G22*H22</f>
+        <v/>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>stehend</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>TPU 95A</t>
-        </is>
-      </c>
+      <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n"/>
       <c r="C23" s="3" t="n"/>
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I23" s="13">
-        <f>SUMIFS(I2:I19,C2:C19,A23)</f>
-        <v/>
-      </c>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>PLA</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Summe nach Material</t>
         </is>
       </c>
       <c r="B24" s="3" t="n"/>
@@ -4038,22 +4151,15 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I24" s="13">
-        <f>SUMIFS(I2:I19,C2:C19,A24)</f>
-        <v/>
-      </c>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Alle Druckteile</t>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
         </is>
       </c>
       <c r="B25" s="3" t="n"/>
@@ -4062,13 +4168,85 @@
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="14">
-        <f>SUM(I22:I24)</f>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I25" s="13">
+        <f>SUMIFS(I2:I22,C2:C22,A25)</f>
         <v/>
       </c>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>TPU 95A</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I26" s="13">
+        <f>SUMIFS(I2:I22,C2:C22,A26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>PLA</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n"/>
+      <c r="C27" s="3" t="n"/>
+      <c r="D27" s="3" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I27" s="13">
+        <f>SUMIFS(I2:I22,C2:C22,A27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="3" t="n"/>
+      <c r="K27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Alle Druckteile</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="14">
+        <f>SUM(I25:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4113,7 +4291,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Druckteile!I25</f>
+        <f>Druckteile!I28</f>
         <v/>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Baseplate V2.9: printed Pi spacers, driver on 16 mm spacers
- four printed sleeves (d6 x 6, bore 2.8) under the Pi 5; an M2.5x16 from
  below through plate, sleeve and Pi threads into the AI HAT+ standoffs
- driver board height 12 -> 16 mm (spacers supplied with the board),
  clearance to the back shell still 6.6 mm
- STL SLARC_Pi_Sleeve, BOM: M2.5x16 instead of bought Pi standoffs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -2532,19 +2532,19 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x6 (Innen/Innen)</t>
+          <t>Zylinderschraube M2,5x16</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Pi 5 (M2 geht mit Scheiben)</t>
+          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
         <v>4</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G52" s="3">
         <f>E52+F52</f>
@@ -2569,12 +2569,12 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Distanzbolzen M2,5x12 (Innen/Innen)</t>
+          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Treiberboard (Stiftleiste unten 9,4 mm)</t>
+          <t>liegen dem Treiber bei</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
@@ -2592,7 +2592,11 @@
         <f>IF(H53="","",G53*H53)</f>
         <v/>
       </c>
-      <c r="J53" s="10" t="n"/>
+      <c r="J53" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K53" s="10" t="n"/>
     </row>
     <row r="54">
@@ -2611,11 +2615,11 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>für die Distanzbolzen, je 2</t>
+          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
         </is>
       </c>
       <c r="E54" s="7" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F54" s="7" t="n">
         <v>2</v>
@@ -3067,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4127,24 +4131,54 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Distanzhülse Pi</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Baseplate-Makro V2.9 / Pi_Sleeve</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G23" s="12">
+        <f>E23*F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="13">
+        <f>D23*G23*H23</f>
+        <v/>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>stehend</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Summe nach Material</t>
-        </is>
-      </c>
+      <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n"/>
       <c r="C24" s="3" t="n"/>
       <c r="D24" s="3" t="n"/>
@@ -4157,9 +4191,9 @@
       <c r="K24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>PETG</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Summe nach Material</t>
         </is>
       </c>
       <c r="B25" s="3" t="n"/>
@@ -4168,22 +4202,15 @@
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I25" s="13">
-        <f>SUMIFS(I2:I22,C2:C22,A25)</f>
-        <v/>
-      </c>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A</t>
+          <t>PETG</t>
         </is>
       </c>
       <c r="B26" s="3" t="n"/>
@@ -4198,7 +4225,7 @@
         </is>
       </c>
       <c r="I26" s="13">
-        <f>SUMIFS(I2:I22,C2:C22,A26)</f>
+        <f>SUMIFS(I2:I23,C2:C23,A26)</f>
         <v/>
       </c>
       <c r="J26" s="3" t="n"/>
@@ -4207,7 +4234,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>PLA</t>
+          <t>TPU 95A</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -4222,16 +4249,16 @@
         </is>
       </c>
       <c r="I27" s="13">
-        <f>SUMIFS(I2:I22,C2:C22,A27)</f>
+        <f>SUMIFS(I2:I23,C2:C23,A27)</f>
         <v/>
       </c>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Alle Druckteile</t>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>PLA</t>
         </is>
       </c>
       <c r="B28" s="3" t="n"/>
@@ -4240,13 +4267,37 @@
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="14">
-        <f>SUM(I25:I27)</f>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I28" s="13">
+        <f>SUMIFS(I2:I23,C2:C23,A28)</f>
         <v/>
       </c>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Alle Druckteile</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
+      <c r="I29" s="14">
+        <f>SUM(I26:I28)</f>
+        <v/>
+      </c>
+      <c r="J29" s="3" t="n"/>
+      <c r="K29" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4291,7 +4342,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Druckteile!I28</f>
+        <f>Druckteile!I29</f>
         <v/>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Power button with ESP32 deep sleep (Baseplate V2.10)
- 12 mm panel push button at the rear right between the plates, recessed
  5 mm behind the plate edge, printed bracket with 1x M3 on the bottom plate
- hub board: J6 button, R7 10k pull-up, J7 -> IO35 (deep-sleep wake-up)
- power sequence: battery stays connected; button wakes / switches off,
  web shutdown via the Pi, 5 s hold = emergency stop; storage: unplug
  Deans + balancer at the rear holder
- interface doc: IO35, sequence, protocol needs, watchdog, open items
  (measure deep-sleep current; fallback K8 self-hold)
- BOM: button, 10k x7, M3, bracket; STL SLARC_Button_Bracket

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -602,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -977,24 +977,24 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Steuerung</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Widerstand 10 kΩ</t>
+          <t>Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>externe Pull-ups Fußkontakte (lange Kabel)</t>
+          <t>Ein/Aus: weckt ESP32 aus dem Deep Sleep (IO35), kurz = aus, 5 s = Notaus; Gewindelänge &gt;= 6 mm, Kopf-Ø &lt;= 15 mm</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3">
         <f>E10+F10</f>
@@ -1019,19 +1019,19 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>WS2812B-LED-Streifen (optional)</t>
+          <t>Widerstand 10 kΩ</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Daten an IO4; 5 V vom Treiber (bis ~10 LEDs) oder vom DC-DC</t>
+          <t>Pull-ups Fußkontakte (6) + Ein/Aus-Taster an IO35 (1)</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G11" s="3">
         <f>E11+F11</f>
@@ -1051,21 +1051,21 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Sensorik</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
+          <t>WS2812B-LED-Streifen (optional)</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>39x39 mm, M12-Halter</t>
+          <t>Daten an IO4; 5 V vom Treiber (bis ~10 LEDs) oder vom DC-DC</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>0</v>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
+          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>F2.2, 1/2.7"</t>
+          <t>39x39 mm, M12-Halter</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
+          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Kamera -&gt; Pi 5 CAM0/CAM1</t>
+          <t>F2.2, 1/2.7"</t>
         </is>
       </c>
       <c r="E14" s="7" t="n">
@@ -1167,16 +1167,16 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Verteilerplatine</t>
+          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Eigenbau, 20x22 mm</t>
+          <t>Kamera -&gt; Pi 5 CAM0/CAM1</t>
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>0</v>
@@ -1204,19 +1204,19 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Mikroschalter D2F (oder ähnlich)</t>
+          <t>Trigger-Verteilerplatine</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Fußkontakt; Maße im Bein-Makro (sw_*) anpassen</t>
+          <t>Eigenbau, 20x22 mm</t>
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" s="3">
         <f>E16+F16</f>
@@ -1236,24 +1236,24 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Sensorik</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>LiPo ZEEE 3S 9000 mAh</t>
+          <t>Mikroschalter D2F (oder ähnlich)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>ca. 170x50x32 mm, Deans (Buchse am Akku)</t>
+          <t>Fußkontakt; Maße im Bein-Makro (sw_*) anpassen</t>
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17" s="3">
         <f>E17+F17</f>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
+          <t>LiPo ZEEE 3S 9000 mAh</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>kleineres BMS reicht (Mittel ~10 A, Spitzen 20–30 A)</t>
+          <t>ca. 170x50x32 mm, Deans (Buchse am Akku)</t>
         </is>
       </c>
       <c r="E18" s="7" t="n">
@@ -1315,19 +1315,19 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Flachsicherung 30–40 A + Halter</t>
+          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>direkt am Akku</t>
+          <t>kleineres BMS reicht (Mittel ~10 A, Spitzen 20–30 A)</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" s="3">
         <f>E19+F19</f>
@@ -1352,19 +1352,19 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Relaismodul 8-Kanal</t>
+          <t>Flachsicherung 30–40 A + Halter</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>8× SRD-05VDC-SL-C (10 A): K1 12 V -&gt; DC-DC (Pi), K2–K7 je ein Bein, K8 frei; Jumper JD-VCC ziehen (VCC 3,3 V, JD-VCC 5 V)</t>
+          <t>direkt am Akku</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="3">
         <f>E20+F20</f>
@@ -1389,19 +1389,19 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
+          <t>Relaismodul 8-Kanal</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Gegenstück zur Deans-Buchse am Akku; sitzt im Steckerhalter (untere Platte hinten)</t>
+          <t>8× SRD-05VDC-SL-C (10 A): K1 12 V -&gt; DC-DC (Pi), K2–K7 je ein Bein, K8 frei; Jumper JD-VCC ziehen (VCC 3,3 V, JD-VCC 5 V)</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3">
         <f>E21+F21</f>
@@ -1426,19 +1426,19 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Litze AWG20 rot/schwarz (m)</t>
+          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>vorhanden; je Bein 12 V (von Kx NO) + GND, Relais-COM, DC-DC, Pi-5V (je Pol 2 Adern)</t>
+          <t>Gegenstück zur Deans-Buchse am Akku; sitzt im Steckerhalter (untere Platte hinten)</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22" s="3">
         <f>E22+F22</f>
@@ -1458,24 +1458,24 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Bein-Platine A (Lochraster ½ 3×7 cm)</t>
+          <t>Litze AWG20 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Eigenbau, Layout Documentation/Wiring</t>
+          <t>vorhanden; je Bein 12 V (von Kx NO) + GND, Relais-COM, DC-DC, Pi-5V (je Pol 2 Adern)</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3">
         <f>E23+F23</f>
@@ -1500,15 +1500,19 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n"/>
+          <t>Bein-Platine A (Lochraster ½ 3×7 cm)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Eigenbau, Layout Documentation/Wiring</t>
+        </is>
+      </c>
       <c r="E24" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="3">
         <f>E24+F24</f>
@@ -1533,19 +1537,15 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Dupont-Kabel (Trigger/Strobe)</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Kameras &lt;-&gt; Trigger-Platine</t>
-        </is>
-      </c>
+          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n"/>
       <c r="E25" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="3">
         <f>E25+F25</f>
@@ -1570,16 +1570,16 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
+          <t>Dupont-Kabel (Trigger/Strobe)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>je Bein-Platine, + an 12 V</t>
+          <t>Kameras &lt;-&gt; Trigger-Platine</t>
         </is>
       </c>
       <c r="E26" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F26" s="7" t="n">
         <v>2</v>
@@ -1607,19 +1607,19 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Keramikkondensator 100 nF</t>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Abblockung MCP23017 (Hub)</t>
+          <t>je Bein-Platine, + an 12 V</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G27" s="3">
         <f>E27+F27</f>
@@ -1644,19 +1644,19 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Transistor BC547 (NPN)</t>
+          <t>Keramikkondensator 100 nF</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
+          <t>Abblockung MCP23017 (Hub)</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G28" s="3">
         <f>E28+F28</f>
@@ -1681,19 +1681,19 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Widerstand 4,7 kΩ</t>
+          <t>Transistor BC547 (NPN)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Basiswiderstand BC547</t>
+          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G29" s="3">
         <f>E29+F29</f>
@@ -1718,19 +1718,19 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
+          <t>Widerstand 4,7 kΩ</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
+          <t>Basiswiderstand BC547</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F30" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G30" s="3">
         <f>E30+F30</f>
@@ -1755,16 +1755,16 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter auf die Eingangsstifte des Relaismoduls (nur ~16 mm Höhe frei)</t>
+          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="7" t="n">
         <v>0</v>
@@ -1792,12 +1792,12 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Lochrasterplatinen AZ-Delivery</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
+          <t>Relais-Adapter auf die Eingangsstifte des Relaismoduls (nur ~16 mm Höhe frei)</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
@@ -1829,16 +1829,16 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
+          <t>Lochrasterplatinen AZ-Delivery</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
+          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F33" s="7" t="n">
         <v>0</v>
@@ -1861,21 +1861,21 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Litze AWG14 rot/schwarz (m)</t>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
+          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" s="7" t="n">
         <v>0</v>
@@ -1898,21 +1898,21 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Kupferdraht 1,5 mm² massiv (m)</t>
+          <t>Litze AWG14 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
+          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F35" s="7" t="n">
         <v>0</v>
@@ -1940,16 +1940,16 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Schienen Bein-Platinen und Hub</t>
+          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="F36" s="7" t="n">
         <v>0</v>
@@ -1977,19 +1977,19 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Servokabel 5264 3-pol.</t>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
+          <t>Schienen Bein-Platinen und Hub</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3">
         <f>E37+F37</f>
@@ -2009,24 +2009,24 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
+          <t>Servokabel 5264 3-pol.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
+          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G38" s="3">
         <f>E38+F38</f>
@@ -2051,12 +2051,12 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x6</t>
+          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
@@ -2088,19 +2088,19 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
+          <t>Zylinderschraube M3x6</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
+          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G40" s="3">
         <f>E40+F40</f>
@@ -2125,19 +2125,19 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x50</t>
+          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
+          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" s="3">
         <f>E41+F41</f>
@@ -2162,19 +2162,19 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
+          <t>Zylinderschraube M3x50</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>unten in den 6 Panzersäulen</t>
+          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G42" s="3">
         <f>E42+F42</f>
@@ -2199,19 +2199,19 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
+          <t>unten in den 6 Panzersäulen</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F43" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F43" s="7" t="n">
-        <v>1</v>
       </c>
       <c r="G43" s="3">
         <f>E43+F43</f>
@@ -2236,16 +2236,16 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12 + Mutter</t>
+          <t>Zylinderschraube M3x45</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" s="7" t="n">
         <v>1</v>
@@ -2273,19 +2273,19 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G45" s="3">
         <f>E45+F45</f>
@@ -2310,19 +2310,19 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Säulen + Stoß + Relais</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G46" s="3">
         <f>E46+F46</f>
@@ -2347,19 +2347,19 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Säulen + Stoß + Relais</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F47" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="F47" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G47" s="3">
         <f>E47+F47</f>
@@ -2384,19 +2384,19 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Zylinderschraube M3x14</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Hub-Träger auf Modulplatz MCP (2) + Steckerhalter Akku (2)</t>
+          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G48" s="3">
         <f>E48+F48</f>
@@ -2421,16 +2421,16 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>DC-DC-Laschen (2) + Hub-Träger (2) + Steckerhalter Akku (2) + Taster-Winkel (1)</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F49" s="7" t="n">
         <v>2</v>
@@ -2458,19 +2458,19 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x5</t>
+          <t>Zylinderschraube M2x6</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Lochraster-Platinen: 6× Bein (je 2), Hub (4), Power-Verteiler (2), direkt ins 1,7-mm-Kernloch</t>
+          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G50" s="3">
         <f>E50+F50</f>
@@ -2495,19 +2495,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Zylinderschraube M2x5</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>Lochraster-Platinen: 6× Bein (je 2), Hub (4), Power-Verteiler (2), direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G51" s="3">
         <f>E51+F51</f>
@@ -2532,19 +2532,19 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x16</t>
+          <t>Zylinderschraube M2x25 + Mutter</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G52" s="3">
         <f>E52+F52</f>
@@ -2569,19 +2569,19 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
+          <t>Zylinderschraube M2,5x16</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>liegen dem Treiber bei</t>
+          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
         <v>4</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G53" s="3">
         <f>E53+F53</f>
@@ -2592,11 +2592,7 @@
         <f>IF(H53="","",G53*H53)</f>
         <v/>
       </c>
-      <c r="J53" s="10" t="inlineStr">
-        <is>
-          <t>vorhanden</t>
-        </is>
-      </c>
+      <c r="J53" s="10" t="n"/>
       <c r="K53" s="10" t="n"/>
     </row>
     <row r="54">
@@ -2610,19 +2606,19 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
+          <t>liegen dem Treiber bei</t>
         </is>
       </c>
       <c r="E54" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G54" s="3">
         <f>E54+F54</f>
@@ -2633,7 +2629,11 @@
         <f>IF(H54="","",G54*H54)</f>
         <v/>
       </c>
-      <c r="J54" s="10" t="n"/>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K54" s="10" t="n"/>
     </row>
     <row r="55">
@@ -2647,15 +2647,19 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="n"/>
+          <t>Zylinderschraube M2,5x5</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
+        </is>
+      </c>
       <c r="E55" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G55" s="3">
         <f>E55+F55</f>
@@ -2680,14 +2684,10 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n"/>
       <c r="E56" s="7" t="n">
         <v>1</v>
       </c>
@@ -2712,21 +2712,21 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F57" s="7" t="n">
         <v>0</v>
@@ -2754,16 +2754,16 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F58" s="7" t="n">
         <v>0</v>
@@ -2791,12 +2791,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -2865,12 +2865,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
@@ -2897,21 +2897,21 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" s="7" t="n">
         <v>0</v>
@@ -2939,16 +2939,16 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="F63" s="7" t="n">
         <v>0</v>
@@ -2976,16 +2976,16 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>PLA orange (kg)</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="F64" s="7" t="n">
         <v>0</v>
@@ -3003,17 +3003,41 @@
       <c r="K64" s="10" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n"/>
-      <c r="B65" s="3" t="n"/>
-      <c r="C65" s="3" t="n"/>
-      <c r="D65" s="3" t="n"/>
-      <c r="E65" s="3" t="n"/>
-      <c r="F65" s="3" t="n"/>
-      <c r="G65" s="3" t="n"/>
-      <c r="H65" s="3" t="n"/>
-      <c r="I65" s="3" t="n"/>
-      <c r="J65" s="3" t="n"/>
-      <c r="K65" s="3" t="n"/>
+      <c r="A65" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>PLA orange (kg)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F65" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="3">
+        <f>E65+F65</f>
+        <v/>
+      </c>
+      <c r="H65" s="8" t="n"/>
+      <c r="I65" s="9">
+        <f>IF(H65="","",G65*H65)</f>
+        <v/>
+      </c>
+      <c r="J65" s="10" t="n"/>
+      <c r="K65" s="10" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -3023,15 +3047,8 @@
       <c r="E66" s="3" t="n"/>
       <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="n"/>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I66" s="11">
-        <f>SUM(I2:I64)</f>
-        <v/>
-      </c>
+      <c r="H66" s="3" t="n"/>
+      <c r="I66" s="3" t="n"/>
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="3" t="n"/>
     </row>
@@ -3043,21 +3060,41 @@
       <c r="E67" s="3" t="n"/>
       <c r="F67" s="3" t="n"/>
       <c r="G67" s="3" t="n"/>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I67" s="3">
-        <f>COUNT(H2:H64)&amp;" von 63"</f>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I67" s="11">
+        <f>SUM(I2:I65)</f>
         <v/>
       </c>
       <c r="J67" s="3" t="n"/>
       <c r="K67" s="3" t="n"/>
     </row>
+    <row r="68">
+      <c r="A68" s="3" t="n"/>
+      <c r="B68" s="3" t="n"/>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I68" s="3">
+        <f>COUNT(H2:H65)&amp;" von 64"</f>
+        <v/>
+      </c>
+      <c r="J68" s="3" t="n"/>
+      <c r="K68" s="3" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3071,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3727,7 +3764,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>87.75</v>
+        <v>87.70999999999999</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>1.27</v>
@@ -4178,24 +4215,54 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Taster-Winkel</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Baseplate-Makro V2.10 / Button_Bracket</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G24" s="12">
+        <f>E24*F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="13">
+        <f>D24*G24*H24</f>
+        <v/>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Fuß aufs Bett, Blende stehend</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Summe nach Material</t>
-        </is>
-      </c>
+      <c r="A25" s="3" t="n"/>
       <c r="B25" s="3" t="n"/>
       <c r="C25" s="3" t="n"/>
       <c r="D25" s="3" t="n"/>
@@ -4208,9 +4275,9 @@
       <c r="K25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>PETG</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Summe nach Material</t>
         </is>
       </c>
       <c r="B26" s="3" t="n"/>
@@ -4219,22 +4286,15 @@
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I26" s="13">
-        <f>SUMIFS(I2:I23,C2:C23,A26)</f>
-        <v/>
-      </c>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A</t>
+          <t>PETG</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -4249,7 +4309,7 @@
         </is>
       </c>
       <c r="I27" s="13">
-        <f>SUMIFS(I2:I23,C2:C23,A27)</f>
+        <f>SUMIFS(I2:I24,C2:C24,A27)</f>
         <v/>
       </c>
       <c r="J27" s="3" t="n"/>
@@ -4258,7 +4318,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>PLA</t>
+          <t>TPU 95A</t>
         </is>
       </c>
       <c r="B28" s="3" t="n"/>
@@ -4273,16 +4333,16 @@
         </is>
       </c>
       <c r="I28" s="13">
-        <f>SUMIFS(I2:I23,C2:C23,A28)</f>
+        <f>SUMIFS(I2:I24,C2:C24,A28)</f>
         <v/>
       </c>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Alle Druckteile</t>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>PLA</t>
         </is>
       </c>
       <c r="B29" s="3" t="n"/>
@@ -4291,13 +4351,37 @@
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
       <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="14">
-        <f>SUM(I26:I28)</f>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I29" s="13">
+        <f>SUMIFS(I2:I24,C2:C24,A29)</f>
         <v/>
       </c>
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Alle Druckteile</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="14">
+        <f>SUM(I27:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4342,7 +4426,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Druckteile!I29</f>
+        <f>Druckteile!I30</f>
         <v/>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
BOM: print settings per part and per material
- Druckteile: columns for walls, orientation and supports/notes; infill
  updated (plates 40 %), ST3215 dummy as optional row
- new sheet Druckeinstellungen with the settings shared by all parts of a
  material (PETG, TPU 95A, PLA): temperatures, fan, first layer, holes,
  retract, bridges, walls, top/bottom, adhesion

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -9,7 +9,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaufteile" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Druckteile" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gewicht" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Druckeinstellungen" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gewicht" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -99,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +121,12 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -500,8 +507,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="3" t="n"/>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Druckeinstellungen</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Blatt Druckeinstellungen: Werte, die für alle Teile eines Materials gelten. Teilespezifisches (Füllung, Wände, Ausrichtung, Stützen) im Blatt Druckteile.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -3108,7 +3123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3120,7 +3135,9 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="52" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3176,7 +3193,17 @@
       </c>
       <c r="K1" s="6" t="inlineStr">
         <is>
-          <t>Druckausrichtung / Hinweis</t>
+          <t>Wände (Linien à 0,4)</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>Druckausrichtung</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Stützen / Besonderes</t>
         </is>
       </c>
     </row>
@@ -3221,9 +3248,17 @@
           <t>50 % Gyroid</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Gelenkachse senkrecht, Tree Support</t>
+      <c r="K2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Gelenkachse senkrecht</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Tree Support</t>
         </is>
       </c>
     </row>
@@ -3268,9 +3303,17 @@
           <t>50 % Gyroid</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>wie rechts</t>
+      <c r="K3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Gelenkachse senkrecht</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Tree Support</t>
         </is>
       </c>
     </row>
@@ -3312,12 +3355,20 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>40 % Gyroid</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Gelenkachse senkrecht, Tree Support</t>
+          <t>40 % Gyroid (nur Gelenkbereiche)</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Gelenkachse senkrecht</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Tree Support; 5 Wände = 2-mm-Rohrwand; Brückeneinstellungen an (16-mm-Decke im Rohr)</t>
         </is>
       </c>
     </row>
@@ -3359,12 +3410,20 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>40 % Gyroid</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>wie rechts</t>
+          <t>40 % Gyroid (nur Gelenkbereiche)</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Gelenkachse senkrecht</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Tree Support; Brückeneinstellungen an</t>
         </is>
       </c>
     </row>
@@ -3409,9 +3468,17 @@
           <t>40 % Gyroid</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Gelenkachse senkrecht, Tree Support</t>
+      <c r="K6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>Gelenkachse senkrecht</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Tree Support; Brückeneinstellungen an</t>
         </is>
       </c>
     </row>
@@ -3456,9 +3523,17 @@
           <t>40 % Gyroid</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>wie rechts</t>
+      <c r="K7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Gelenkachse senkrecht</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Tree Support; Brückeneinstellungen an</t>
         </is>
       </c>
     </row>
@@ -3500,12 +3575,20 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>20–25 % Gyroid, 5 Wände</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>Öffnung nach unten, ohne Stützen</t>
+          <t>20–25 % Gyroid</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>Öffnung nach unten</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -3550,9 +3633,17 @@
           <t>20 %</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>flach</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -3597,9 +3688,17 @@
           <t>20 %</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>flach</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -3641,12 +3740,20 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>30 % Gyroid</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>Unterseite aufs Bett, Brim 5 mm</t>
+          <t>40 % Gyroid</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Unterseite aufs Bett</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>keine; Brim 8 mm</t>
         </is>
       </c>
     </row>
@@ -3688,12 +3795,20 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>30 % Gyroid</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>kopfüber drucken (Stoßzunge oben)</t>
+          <t>40 % Gyroid</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Oberseite aufs Bett (Stoßzunge oben flach)</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>keine; Brim 8 mm</t>
         </is>
       </c>
     </row>
@@ -3735,12 +3850,20 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>30 % Gyroid</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>Unterseite aufs Bett (V2.8: M2-Bunde für 4 Bein-Platinen)</t>
+          <t>40 % Gyroid</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Unterseite aufs Bett</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>keine; Brim 8 mm; M2-Bunde für 4 Bein-Platinen</t>
         </is>
       </c>
     </row>
@@ -3782,12 +3905,20 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>30 % Gyroid</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>Stoßzunge braucht flache Stütze</t>
+          <t>40 % Gyroid</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Unterseite aufs Bett</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>flache Stütze nur unter der Stoßzunge (sonst Support-Blocker); Brim 8 mm</t>
         </is>
       </c>
     </row>
@@ -3829,12 +3960,20 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>30 %</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>Frontfläche aufs Bett, Brim 6–8 mm, Lüfter erst ab Schicht 4</t>
+          <t>40 % Gyroid</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Frontfläche aufs Bett</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>keine; Brim 6–8 mm</t>
         </is>
       </c>
     </row>
@@ -3879,9 +4018,17 @@
           <t>100 %</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>Laschen aufs Bett, Tunnel liegen waagrecht (kurze Brücken)</t>
+      <c r="K16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Laschen aufs Bett</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>keine; Tunnel als kurze Brücken</t>
         </is>
       </c>
     </row>
@@ -3923,12 +4070,20 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>100 %, 4 Wände</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>stehend, Kopf aufs Bett, ohne Stützen</t>
+          <t>100 %</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>stehend, Kopf aufs Bett</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -3970,12 +4125,20 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>100 % (Gitter, 4 Wände)</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>Grundfläche aufs Bett, ohne Stützen</t>
+          <t>100 % (Gitter)</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Grundfläche aufs Bett</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>keine; Dachunterseite 50°</t>
         </is>
       </c>
     </row>
@@ -4017,12 +4180,20 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>100 % (Gitter, 4 Wände)</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>Grundfläche aufs Bett, ohne Stützen</t>
+          <t>100 % (Gitter)</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Grundfläche aufs Bett</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>keine; Dachunterseite 50°</t>
         </is>
       </c>
     </row>
@@ -4064,12 +4235,20 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>30 %</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>Bunde nach oben, ohne Stützen</t>
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>flach, Bunde nach oben</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -4111,12 +4290,20 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>30 %</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
+          <t>40 %</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
         <is>
           <t>Deck aufs Bett, Bunde nach oben</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -4161,9 +4348,17 @@
           <t>100 %</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>stehend</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
         </is>
       </c>
     </row>
@@ -4208,9 +4403,17 @@
           <t>100 %</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
         <is>
           <t>stehend</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>keine; Bohrung bei Bedarf auf 2,8–3 mm aufbohren</t>
         </is>
       </c>
     </row>
@@ -4255,31 +4458,77 @@
           <t>100 %</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>Fuß aufs Bett, Blende stehend</t>
         </is>
       </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>ST3215-Dummy (optional)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Drawings/STL files/ST3215_Dummy.stl</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="G25" s="12">
+        <f>E25*F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I25" s="13">
+        <f>D25*G25*H25</f>
+        <v/>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>15 %</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>seitlich liegend</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>keine; Anzahl nach Bedarf eintragen (Platzhalter für fehlende Coxa-Servos)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Summe nach Material</t>
-        </is>
-      </c>
+      <c r="A26" s="3" t="n"/>
       <c r="B26" s="3" t="n"/>
       <c r="C26" s="3" t="n"/>
       <c r="D26" s="3" t="n"/>
@@ -4290,11 +4539,13 @@
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>PETG</t>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Summe nach Material</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -4303,22 +4554,17 @@
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>g gesamt</t>
-        </is>
-      </c>
-      <c r="I27" s="13">
-        <f>SUMIFS(I2:I24,C2:C24,A27)</f>
-        <v/>
-      </c>
+      <c r="H27" s="3" t="n"/>
+      <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="3" t="n"/>
+      <c r="L27" s="3" t="n"/>
+      <c r="M27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A</t>
+          <t>PETG</t>
         </is>
       </c>
       <c r="B28" s="3" t="n"/>
@@ -4333,16 +4579,18 @@
         </is>
       </c>
       <c r="I28" s="13">
-        <f>SUMIFS(I2:I24,C2:C24,A28)</f>
+        <f>SUMIFS(I2:I25,C2:C25,A28)</f>
         <v/>
       </c>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>PLA</t>
+          <t>TPU 95A</t>
         </is>
       </c>
       <c r="B29" s="3" t="n"/>
@@ -4357,16 +4605,18 @@
         </is>
       </c>
       <c r="I29" s="13">
-        <f>SUMIFS(I2:I24,C2:C24,A29)</f>
+        <f>SUMIFS(I2:I25,C2:C25,A29)</f>
         <v/>
       </c>
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="3" t="n"/>
+      <c r="L29" s="3" t="n"/>
+      <c r="M29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Alle Druckteile</t>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>PLA</t>
         </is>
       </c>
       <c r="B30" s="3" t="n"/>
@@ -4375,13 +4625,41 @@
       <c r="E30" s="3" t="n"/>
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="14">
-        <f>SUM(I27:I29)</f>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>g gesamt</t>
+        </is>
+      </c>
+      <c r="I30" s="13">
+        <f>SUMIFS(I2:I25,C2:C25,A30)</f>
         <v/>
       </c>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Alle Druckteile</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n"/>
+      <c r="C31" s="3" t="n"/>
+      <c r="D31" s="3" t="n"/>
+      <c r="E31" s="3" t="n"/>
+      <c r="F31" s="3" t="n"/>
+      <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="n"/>
+      <c r="I31" s="14">
+        <f>SUM(I28:I30)</f>
+        <v/>
+      </c>
+      <c r="J31" s="3" t="n"/>
+      <c r="K31" s="3" t="n"/>
+      <c r="L31" s="3" t="n"/>
+      <c r="M31" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4389,6 +4667,400 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Einstellung</t>
+        </is>
+      </c>
+      <c r="B1" s="18" t="inlineStr">
+        <is>
+          <t>PETG</t>
+        </is>
+      </c>
+      <c r="C1" s="18" t="inlineStr">
+        <is>
+          <t>TPU 95A</t>
+        </is>
+      </c>
+      <c r="D1" s="18" t="inlineStr">
+        <is>
+          <t>PLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Düse</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>0,4 mm</t>
+        </is>
+      </c>
+      <c r="C2" s="19" t="inlineStr">
+        <is>
+          <t>0,4 mm</t>
+        </is>
+      </c>
+      <c r="D2" s="19" t="inlineStr">
+        <is>
+          <t>0,4 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Schichthöhe</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>0,2 mm (erste Schicht 0,2–0,24 mm)</t>
+        </is>
+      </c>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>0,2 mm</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>0,2 mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Düsentemperatur</t>
+        </is>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>235 °C</t>
+        </is>
+      </c>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>225 °C</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>210 °C</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Betttemperatur</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>80 °C, große flache Teile 85 °C</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>50 °C</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>60 °C</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Lüfter</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>erste 3–4 Schichten aus, danach max. 30–40 %</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>50 %</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>100 % ab Schicht 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Druckgeschwindigkeit</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>normal; erste Schicht 20 mm/s</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>20–25 mm/s</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Erste Schicht</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Linienbreite 120 %, horizontale Ausdehnung −0,1 mm (Elefantenfuß)</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Linienbreite 120 %</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Linienbreite 120 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>Löcher</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>horizontale Ausdehnung für Löcher +0,1 mm, falls M2/M2,5/M3 zu eng</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Rückzug (Retract)</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>kurz (≤ 1 mm) oder aus</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>Brücken</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Brückeneinstellungen an: Wand/Haut 20–25 mm/s, Lüfter Brücke 100 %, Haut-Fluss 100 % (bei Durchhängen 90 %), mehrere Brückenschichten an</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>Wände (Standard)</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>4 Linien (1,6 mm); Bein-Rohre 5 Linien = 2 mm</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>5 Linien</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>2 Linien</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>Deck-/Bodenschichten</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>je 5 (1 mm)</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>je 4</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>je 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Haftung</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Brim bei großen flachen Teilen (Platten 8 mm, Kamerahalter 6–8 mm), sonst keine</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Umgebung</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>kein Luftzug; Teil auf dem Bett abkühlen lassen</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Kernlöcher</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>M2 = 1,7 mm, M2,5 = 2,1 mm: Wandzahl ist wichtiger als Füllung</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Kleinteile</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>mehrere 100-%-Teile zusammen auf eine Platte (Kühlzeit je Schicht)</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4426,7 +5098,7 @@
         </is>
       </c>
       <c r="B2" s="15">
-        <f>Druckteile!I30</f>
+        <f>Druckteile!I31</f>
         <v/>
       </c>
       <c r="C2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
BOM: order list for screws and electronics
- new sheet Bestellliste: screws/nuts/inserts sorted by thread and length,
  electronics grouped; quantities incl. reserve via SUMIF from Kaufteile,
  status via INDEX/MATCH
- fixes: camera bracket ears are M3 (M3x25 + nut, not M2x25); lock nuts
  14 (+4) after the threaded inserts; fuse row = 30 A + inline holder
- ICM-20948 added (on hand); spring wire usage described; known stock
  marked as vorhanden

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -8,9 +8,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kaufteile" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Druckteile" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Druckeinstellungen" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gewicht" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bestellliste" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Druckteile" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Druckeinstellungen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gewicht" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00\ &quot;€&quot;;\-#,##0.00\ &quot;€&quot;;\-"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +70,13 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -100,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,6 +135,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -555,8 +565,16 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="3" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Bestellliste</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Blatt Bestellliste: Schrauben und Elektronik geordnet, Mengen inkl. Reserve per Formel aus Kaufteile, Status ebenfalls aus Kaufteile.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -617,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K68"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -761,7 +779,11 @@
         <f>IF(H3="","",G3*H3)</f>
         <v/>
       </c>
-      <c r="J3" s="10" t="n"/>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K3" s="10" t="n"/>
     </row>
     <row r="4">
@@ -835,7 +857,11 @@
         <f>IF(H5="","",G5*H5)</f>
         <v/>
       </c>
-      <c r="J5" s="10" t="n"/>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K5" s="10" t="n"/>
     </row>
     <row r="6">
@@ -872,7 +898,11 @@
         <f>IF(H6="","",G6*H6)</f>
         <v/>
       </c>
-      <c r="J6" s="10" t="n"/>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K6" s="10" t="n"/>
     </row>
     <row r="7">
@@ -1131,7 +1161,11 @@
         <f>IF(H13="","",G13*H13)</f>
         <v/>
       </c>
-      <c r="J13" s="10" t="n"/>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K13" s="10" t="n"/>
     </row>
     <row r="14">
@@ -1288,17 +1322,17 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Sensorik</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>LiPo ZEEE 3S 9000 mAh</t>
+          <t>IMU ICM-20948 (Pimoroni-Breakout)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>ca. 170x50x32 mm, Deans (Buchse am Akku)</t>
+          <t>vorhanden (vom alten Kameramodul); oben auf dem Kamerahalter, I²C am Pi</t>
         </is>
       </c>
       <c r="E18" s="7" t="n">
@@ -1316,7 +1350,11 @@
         <f>IF(H18="","",G18*H18)</f>
         <v/>
       </c>
-      <c r="J18" s="10" t="n"/>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K18" s="10" t="n"/>
     </row>
     <row r="19">
@@ -1330,12 +1368,12 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
+          <t>LiPo ZEEE 3S 9000 mAh</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>kleineres BMS reicht (Mittel ~10 A, Spitzen 20–30 A)</t>
+          <t>ca. 170x50x32 mm, Deans (Buchse am Akku)</t>
         </is>
       </c>
       <c r="E19" s="7" t="n">
@@ -1353,7 +1391,11 @@
         <f>IF(H19="","",G19*H19)</f>
         <v/>
       </c>
-      <c r="J19" s="10" t="n"/>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K19" s="10" t="n"/>
     </row>
     <row r="20">
@@ -1367,19 +1409,19 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Flachsicherung 30–40 A + Halter</t>
+          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>direkt am Akku</t>
+          <t>kleineres BMS reicht (Mittel ~10 A, Spitzen 20–30 A)</t>
         </is>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G20" s="3">
         <f>E20+F20</f>
@@ -1404,19 +1446,19 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Relaismodul 8-Kanal</t>
+          <t>Flachsicherung 30 A + Inline-Halter</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>8× SRD-05VDC-SL-C (10 A): K1 12 V -&gt; DC-DC (Pi), K2–K7 je ein Bein, K8 frei; Jumper JD-VCC ziehen (VCC 3,3 V, JD-VCC 5 V)</t>
+          <t>F1 in der Plusleitung Deans -&gt; Power-Board; Standard-Flachsicherung (ATO), Halter mit Litze ≥ AWG14 (z. B. Neuftech 30 A wasserdicht); Reserve = Ersatzsicherung gleicher Bauform</t>
         </is>
       </c>
       <c r="E21" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" s="3">
         <f>E21+F21</f>
@@ -1441,19 +1483,19 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
+          <t>Relaismodul 8-Kanal</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Gegenstück zur Deans-Buchse am Akku; sitzt im Steckerhalter (untere Platte hinten)</t>
+          <t>8× SRD-05VDC-SL-C (10 A): K1 12 V -&gt; DC-DC (Pi), K2–K7 je ein Bein, K8 frei; Jumper JD-VCC ziehen (VCC 3,3 V, JD-VCC 5 V)</t>
         </is>
       </c>
       <c r="E22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="3">
         <f>E22+F22</f>
@@ -1464,7 +1506,11 @@
         <f>IF(H22="","",G22*H22)</f>
         <v/>
       </c>
-      <c r="J22" s="10" t="n"/>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K22" s="10" t="n"/>
     </row>
     <row r="23">
@@ -1478,19 +1524,19 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Litze AWG20 rot/schwarz (m)</t>
+          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>vorhanden; je Bein 12 V (von Kx NO) + GND, Relais-COM, DC-DC, Pi-5V (je Pol 2 Adern)</t>
+          <t>Gegenstück zur Deans-Buchse am Akku; sitzt im Steckerhalter (untere Platte hinten)</t>
         </is>
       </c>
       <c r="E23" s="7" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="3">
         <f>E23+F23</f>
@@ -1510,24 +1556,24 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Bein-Platine A (Lochraster ½ 3×7 cm)</t>
+          <t>Litze AWG20 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Eigenbau, Layout Documentation/Wiring</t>
+          <t>vorhanden; je Bein 12 V (von Kx NO) + GND, Relais-COM, DC-DC, Pi-5V (je Pol 2 Adern)</t>
         </is>
       </c>
       <c r="E24" s="7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="3">
         <f>E24+F24</f>
@@ -1538,7 +1584,11 @@
         <f>IF(H24="","",G24*H24)</f>
         <v/>
       </c>
-      <c r="J24" s="10" t="n"/>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K24" s="10" t="n"/>
     </row>
     <row r="25">
@@ -1552,15 +1602,19 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n"/>
+          <t>Bein-Platine A (Lochraster ½ 3×7 cm)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Eigenbau, Layout Documentation/Wiring</t>
+        </is>
+      </c>
       <c r="E25" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F25" s="7" t="n">
         <v>1</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G25" s="3">
         <f>E25+F25</f>
@@ -1585,19 +1639,15 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Dupont-Kabel (Trigger/Strobe)</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Kameras &lt;-&gt; Trigger-Platine</t>
-        </is>
-      </c>
+          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n"/>
       <c r="E26" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="3">
         <f>E26+F26</f>
@@ -1622,16 +1672,16 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
+          <t>Dupont-Kabel (Trigger/Strobe)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>je Bein-Platine, + an 12 V</t>
+          <t>Kameras &lt;-&gt; Trigger-Platine</t>
         </is>
       </c>
       <c r="E27" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F27" s="7" t="n">
         <v>2</v>
@@ -1659,19 +1709,19 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Keramikkondensator 100 nF</t>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Abblockung MCP23017 (Hub)</t>
+          <t>je Bein-Platine, + an 12 V</t>
         </is>
       </c>
       <c r="E28" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G28" s="3">
         <f>E28+F28</f>
@@ -1696,19 +1746,19 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Transistor BC547 (NPN)</t>
+          <t>Keramikkondensator 100 nF</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
+          <t>Abblockung MCP23017 (Hub)</t>
         </is>
       </c>
       <c r="E29" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G29" s="3">
         <f>E29+F29</f>
@@ -1733,19 +1783,19 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Widerstand 4,7 kΩ</t>
+          <t>Transistor BC547 (NPN)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Basiswiderstand BC547</t>
+          <t>Relais-Adapter: Pi hält K1 (Diode ginge nicht, ausgeschalteter Pi zieht den Eingang)</t>
         </is>
       </c>
       <c r="E30" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" s="3">
         <f>E30+F30</f>
@@ -1770,19 +1820,19 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
+          <t>Widerstand 4,7 kΩ</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
+          <t>Basiswiderstand BC547</t>
         </is>
       </c>
       <c r="E31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F31" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G31" s="3">
         <f>E31+F31</f>
@@ -1807,16 +1857,16 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Relais-Adapter auf die Eingangsstifte des Relaismoduls (nur ~16 mm Höhe frei)</t>
+          <t>Servo-Anschlüsse Bein-Platinen (18× 3-pol.)</t>
         </is>
       </c>
       <c r="E32" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" s="7" t="n">
         <v>0</v>
@@ -1844,12 +1894,12 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Lochrasterplatinen AZ-Delivery</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
+          <t>Relais-Adapter auf die Eingangsstifte des Relaismoduls (nur ~16 mm Höhe frei)</t>
         </is>
       </c>
       <c r="E33" s="7" t="n">
@@ -1881,16 +1931,16 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
+          <t>Lochrasterplatinen AZ-Delivery</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
+          <t>vorhanden: 3× 3×7 (6 Bein-Platinen), 2× 5×7 (Hub, Power), 1× 2×8 (Relais-Adapter)</t>
         </is>
       </c>
       <c r="E34" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F34" s="7" t="n">
         <v>0</v>
@@ -1904,7 +1954,11 @@
         <f>IF(H34="","",G34*H34)</f>
         <v/>
       </c>
-      <c r="J34" s="10" t="n"/>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K34" s="10" t="n"/>
     </row>
     <row r="35">
@@ -1913,21 +1967,21 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Litze AWG14 rot/schwarz (m)</t>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
+          <t>für XH-Crimps (AWG20 passt nicht in XH-Kontakte): Hub &lt;-&gt; Beine, I²C, INT, Relais</t>
         </is>
       </c>
       <c r="E35" s="7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" s="7" t="n">
         <v>0</v>
@@ -1950,21 +2004,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Verdrahtung</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Kupferdraht 1,5 mm² massiv (m)</t>
+          <t>Litze AWG14 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
+          <t>Akku -&gt; Sicherung -&gt; Power-Board, Akku- -&gt; BMS -&gt; Power-Board; alternativ 3× AWG20 parallel</t>
         </is>
       </c>
       <c r="E36" s="7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F36" s="7" t="n">
         <v>0</v>
@@ -1992,16 +2046,16 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Schienen Bein-Platinen und Hub</t>
+          <t>Sammelschienen Power-Board (z. B. NYM-Rest)</t>
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="F37" s="7" t="n">
         <v>0</v>
@@ -2029,19 +2083,19 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Servokabel 5264 3-pol.</t>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
+          <t>Schienen Bein-Platinen und Hub</t>
         </is>
       </c>
       <c r="E38" s="7" t="n">
         <v>2</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" s="3">
         <f>E38+F38</f>
@@ -2061,24 +2115,24 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Verdrahtung</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
+          <t>Servokabel 5264 3-pol.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
+          <t>H5 -&gt; Hub (nur DATA + GND), ggf. Verlängerung Tibia-Servo</t>
         </is>
       </c>
       <c r="E39" s="7" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G39" s="3">
         <f>E39+F39</f>
@@ -2103,12 +2157,12 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x6</t>
+          <t>Zylinderschraube M3x8 (ISO 7380/4762)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk; NICHT länger (Servogehäuse)</t>
         </is>
       </c>
       <c r="E40" s="7" t="n">
@@ -2140,19 +2194,19 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
+          <t>Zylinderschraube M3x6</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
+          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G41" s="3">
         <f>E41+F41</f>
@@ -2177,19 +2231,19 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x50</t>
+          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
+          <t>Coxa 4 je Servo (Platten), Bein-Servos 2 je Servo</t>
         </is>
       </c>
       <c r="E42" s="7" t="n">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="F42" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G42" s="3">
         <f>E42+F42</f>
@@ -2214,19 +2268,19 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
+          <t>Zylinderschraube M3x50</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>unten in den 6 Panzersäulen</t>
+          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G43" s="3">
         <f>E43+F43</f>
@@ -2251,19 +2305,19 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
+          <t>unten in den 6 Panzersäulen</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F44" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F44" s="7" t="n">
-        <v>1</v>
       </c>
       <c r="G44" s="3">
         <f>E44+F44</f>
@@ -2288,16 +2342,16 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12 + Mutter</t>
+          <t>Zylinderschraube M3x45</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" s="7" t="n">
         <v>1</v>
@@ -2325,19 +2379,19 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" s="3">
         <f>E46+F46</f>
@@ -2362,19 +2416,19 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Säulen + Stoß + Relais</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G47" s="3">
         <f>E47+F47</f>
@@ -2399,19 +2453,19 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Plattenstoß (8) + 2 Säulen M3x45 (2) + Relais (4)</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F48" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="F48" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G48" s="3">
         <f>E48+F48</f>
@@ -2436,19 +2490,19 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Zylinderschraube M3x14</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Hub-Träger (2) + Steckerhalter Akku (2) + Taster-Winkel (1)</t>
+          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F49" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G49" s="3">
         <f>E49+F49</f>
@@ -2473,16 +2527,16 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>DC-DC-Laschen (2) + Hub-Träger (2) + Steckerhalter Akku (2) + Taster-Winkel (1)</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" s="7" t="n">
         <v>2</v>
@@ -2510,19 +2564,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x5</t>
+          <t>Zylinderschraube M2x6</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Lochraster-Platinen: 6× Bein (je 2), Hub (4), Power-Verteiler (2), direkt ins 1,7-mm-Kernloch</t>
+          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F51" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G51" s="3">
         <f>E51+F51</f>
@@ -2547,19 +2601,19 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x25 + Mutter</t>
+          <t>Zylinderschraube M2x5</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>Lochraster-Platinen: 6× Bein (je 2), Hub (4), Power-Verteiler (2), direkt ins 1,7-mm-Kernloch</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G52" s="3">
         <f>E52+F52</f>
@@ -2584,19 +2638,19 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x16</t>
+          <t>Zylinderschraube M3x25 + Mutter</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte (Bohrung 3,2 = M3)</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G53" s="3">
         <f>E53+F53</f>
@@ -2621,19 +2675,19 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
+          <t>Zylinderschraube M2,5x16</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>liegen dem Treiber bei</t>
+          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
         </is>
       </c>
       <c r="E54" s="7" t="n">
         <v>4</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G54" s="3">
         <f>E54+F54</f>
@@ -2644,11 +2698,7 @@
         <f>IF(H54="","",G54*H54)</f>
         <v/>
       </c>
-      <c r="J54" s="10" t="inlineStr">
-        <is>
-          <t>vorhanden</t>
-        </is>
-      </c>
+      <c r="J54" s="10" t="n"/>
       <c r="K54" s="10" t="n"/>
     </row>
     <row r="55">
@@ -2662,19 +2712,19 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
+          <t>liegen dem Treiber bei</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F55" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G55" s="3">
         <f>E55+F55</f>
@@ -2685,7 +2735,11 @@
         <f>IF(H55="","",G55*H55)</f>
         <v/>
       </c>
-      <c r="J55" s="10" t="n"/>
+      <c r="J55" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K55" s="10" t="n"/>
     </row>
     <row r="56">
@@ -2699,15 +2753,19 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="n"/>
+          <t>Zylinderschraube M2,5x5</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
+        </is>
+      </c>
       <c r="E56" s="7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F56" s="7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G56" s="3">
         <f>E56+F56</f>
@@ -2732,14 +2790,10 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Haltestifte Mikroschalter, bündig abknipsen</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n"/>
       <c r="E57" s="7" t="n">
         <v>1</v>
       </c>
@@ -2764,21 +2818,21 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Verbindung</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Haltestifte Mikroschalter: quer durch Tibia und Schalterlöcher, bündig abknipsen (2 je Fuß); Ersatz: Stahlnagel Ø1,2 oder aufgebogene Büroklammer</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
-        <v>50</v>
+        <v>0.5</v>
       </c>
       <c r="F58" s="7" t="n">
         <v>0</v>
@@ -2806,16 +2860,16 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F59" s="7" t="n">
         <v>0</v>
@@ -2843,12 +2897,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -2880,12 +2934,12 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
@@ -2917,12 +2971,12 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
@@ -2949,21 +3003,21 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" s="7" t="n">
         <v>0</v>
@@ -2991,16 +3045,16 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E64" s="7" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="F64" s="7" t="n">
         <v>0</v>
@@ -3028,16 +3082,16 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>PLA orange (kg)</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E65" s="7" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="F65" s="7" t="n">
         <v>0</v>
@@ -3055,17 +3109,41 @@
       <c r="K65" s="10" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n"/>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="n"/>
-      <c r="I66" s="3" t="n"/>
-      <c r="J66" s="3" t="n"/>
-      <c r="K66" s="3" t="n"/>
+      <c r="A66" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Filament</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>PLA orange (kg)</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Zierleisten</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F66" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="3">
+        <f>E66+F66</f>
+        <v/>
+      </c>
+      <c r="H66" s="8" t="n"/>
+      <c r="I66" s="9">
+        <f>IF(H66="","",G66*H66)</f>
+        <v/>
+      </c>
+      <c r="J66" s="10" t="n"/>
+      <c r="K66" s="10" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -3075,15 +3153,8 @@
       <c r="E67" s="3" t="n"/>
       <c r="F67" s="3" t="n"/>
       <c r="G67" s="3" t="n"/>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I67" s="11">
-        <f>SUM(I2:I65)</f>
-        <v/>
-      </c>
+      <c r="H67" s="3" t="n"/>
+      <c r="I67" s="3" t="n"/>
       <c r="J67" s="3" t="n"/>
       <c r="K67" s="3" t="n"/>
     </row>
@@ -3095,21 +3166,41 @@
       <c r="E68" s="3" t="n"/>
       <c r="F68" s="3" t="n"/>
       <c r="G68" s="3" t="n"/>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I68" s="3">
-        <f>COUNT(H2:H65)&amp;" von 64"</f>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I68" s="11">
+        <f>SUM(I2:I66)</f>
         <v/>
       </c>
       <c r="J68" s="3" t="n"/>
       <c r="K68" s="3" t="n"/>
     </row>
+    <row r="69">
+      <c r="A69" s="3" t="n"/>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="3" t="n"/>
+      <c r="D69" s="3" t="n"/>
+      <c r="E69" s="3" t="n"/>
+      <c r="F69" s="3" t="n"/>
+      <c r="G69" s="3" t="n"/>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I69" s="3">
+        <f>COUNT(H2:H66)&amp;" von 65"</f>
+        <v/>
+      </c>
+      <c r="J69" s="3" t="n"/>
+      <c r="K69" s="3" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3118,6 +3209,1448 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Bestellliste – Mengen inkl. Reserve, rechnen aus dem Blatt Kaufteile (Spalte Bestellmenge). Status aus Kaufteile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Schrauben, Muttern, Einsätze</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Gruppe</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Teil</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Bestellmenge</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Verwendung</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Blechschraube</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Blechschraube 2x5 (beiliegend bei ST3215)</t>
+        </is>
+      </c>
+      <c r="C5" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Blechschraube 2x5 (beiliegend bei ST3215)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D5" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Blechschraube 2x5 (beiliegend bei ST3215)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Blechschraube 2x5 (beiliegend bei ST3215)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Coxa-Servos an den Platten (4 je Servo), Bein-Servos unten (2 je Servo); liegen den Servos bei</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M2x5</t>
+        </is>
+      </c>
+      <c r="C6" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2x5",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D6" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x5",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Lochraster-Platinen in 1,7-mm-Kernlöcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M2x6</t>
+        </is>
+      </c>
+      <c r="C7" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2x6",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x6",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Kamera-Platinen in 1,7-mm-Kernlöcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>M2,5</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M2,5x5</t>
+        </is>
+      </c>
+      <c r="C8" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x5",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D8" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Treiber auf Distanzhülsen (nur falls nicht beiliegend)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>M2,5</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M2,5x16</t>
+        </is>
+      </c>
+      <c r="C9" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x16",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D9" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Pi 5 durch Platte + gedruckte Hülse in die HAT-Bolzen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x6</t>
+        </is>
+      </c>
+      <c r="C10" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x6",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D10" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Gabelwange unten -&gt; Servo-Rückscheibe, 4 je Gelenk</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x8</t>
+        </is>
+      </c>
+      <c r="C11" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D11" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x10</t>
+        </is>
+      </c>
+      <c r="C12" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10",Kaufteile!$G:$G)+SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D12" s="19" t="inlineStr"/>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Plattenstoß (8, mit Sicherungsmutter); DC-DC, Hub-Träger, Steckerhalter, Taster-Winkel (7, mit Mutter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x12</t>
+        </is>
+      </c>
+      <c r="C13" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x12 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D13" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Teilungsspant Panzer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x14</t>
+        </is>
+      </c>
+      <c r="C14" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x14",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D14" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x14",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x14",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>Relaismodul auf 5-mm-Bolzen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x25</t>
+        </is>
+      </c>
+      <c r="C15" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x25 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D15" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x45</t>
+        </is>
+      </c>
+      <c r="C16" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x45",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D16" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x45",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x45",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>2 Säulen bei x = -40</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Zylinderschraube M3x50</t>
+        </is>
+      </c>
+      <c r="C17" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x50",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D17" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>6 Säulen unter den Panzersäulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Muttern</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Mutter M3 (DIN 934)</t>
+        </is>
+      </c>
+      <c r="C18" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x*+ Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D18" s="19" t="inlineStr"/>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>zu allen Schrauben „+ Mutter“ (M3x10, M3x12, M3x25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Muttern</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
+        </is>
+      </c>
+      <c r="C19" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Sicherungsmutter M3 (Nylonring)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D19" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Plattenstoß, Säulen M3x45, Relais</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Einsätze</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Gewindeeinsatz M3 (5,7 lang, Ø4,6)</t>
+        </is>
+      </c>
+      <c r="C20" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D20" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Panzersäulen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="C21" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Elektronik isoliert befestigen</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Federstahldraht 1,2 mm (m)</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Federstahldraht 1,2 mm (m)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Haltestifte Mikroschalter</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Elektronik und Verdrahtung</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Gruppe</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Teil</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Bestellmenge</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Verwendung</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Antrieb</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Servo ST3215 (Feetech/Waveshare, 12 V)</t>
+        </is>
+      </c>
+      <c r="C26" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D26" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>18 Servos, 3 je Bein</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Rechner</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 5</t>
+        </is>
+      </c>
+      <c r="C27" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi 5",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D27" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E27" s="19" t="inlineStr">
+        <is>
+          <t>Perzeption, Planung</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Rechner</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Raspberry Pi Active Cooler</t>
+        </is>
+      </c>
+      <c r="C28" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi Active Cooler",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D28" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>falls nicht beim Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>Rechner</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>Hailo-8 AI HAT+ (26 TOPS)</t>
+        </is>
+      </c>
+      <c r="C29" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D29" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>NPU</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Rechner</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Waveshare General Driver for Robots</t>
+        </is>
+      </c>
+      <c r="C30" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Waveshare General Driver for Robots",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D30" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>ESP32, Servo-Bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>LiPo ZEEE 3S 9000 mAh</t>
+        </is>
+      </c>
+      <c r="C31" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"LiPo ZEEE 3S 9000 mAh",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D31" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>Akku</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
+        </is>
+      </c>
+      <c r="C32" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D32" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>Kurzschluss-, Überstrom-, Zellenschutz</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Flachsicherung 30 A + Inline-Halter</t>
+        </is>
+      </c>
+      <c r="C33" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Flachsicherung 30 A + Inline-Halter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D33" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>F1 in der Plusleitung; Inline-Halter, Litze ≥ AWG14</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
+        </is>
+      </c>
+      <c r="C34" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D34" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Steckerhalter</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C</t>
+        </is>
+      </c>
+      <c r="C35" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D35" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>Pi-Versorgung</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Relaismodul 8-Kanal</t>
+        </is>
+      </c>
+      <c r="C36" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Relaismodul 8-Kanal",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D36" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>K1 Pi, K2–K7 Beine</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Sensorik</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
+        </is>
+      </c>
+      <c r="C37" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D37" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>Stereo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>Sensorik</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
+        </is>
+      </c>
+      <c r="C38" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D38" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E38" s="19" t="inlineStr">
+        <is>
+          <t>Stereo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Sensorik</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
+        </is>
+      </c>
+      <c r="C39" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D39" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>Kamera -&gt; Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Sensorik</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>IMU ICM-20948 (Pimoroni-Breakout)</t>
+        </is>
+      </c>
+      <c r="C40" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>VIO/SLAM am Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>Sensorik</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="inlineStr">
+        <is>
+          <t>Mikroschalter D2F (oder ähnlich)</t>
+        </is>
+      </c>
+      <c r="C41" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Mikroschalter D2F (oder ähnlich)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D41" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>Fußkontakte</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>IO-Expander MCP23017-E (Modul/Breakout)</t>
+        </is>
+      </c>
+      <c r="C42" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D42" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>Hub-Platine</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)</t>
+        </is>
+      </c>
+      <c r="C43" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D43" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>Ein/Aus</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="inlineStr">
+        <is>
+          <t>Widerstand 10 kΩ</t>
+        </is>
+      </c>
+      <c r="C44" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 10 kΩ",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D44" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="19" t="inlineStr">
+        <is>
+          <t>Pull-ups Füße + Taster</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="inlineStr">
+        <is>
+          <t>Widerstand 4,7 kΩ</t>
+        </is>
+      </c>
+      <c r="C45" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 4,7 kΩ",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D45" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>Basiswiderstand BC547</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="inlineStr">
+        <is>
+          <t>Transistor BC547 (NPN)</t>
+        </is>
+      </c>
+      <c r="C46" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Transistor BC547 (NPN)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D46" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>Relais-Adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="inlineStr">
+        <is>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
+        </is>
+      </c>
+      <c r="C47" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D47" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>Bein-Platinen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>Bauteile</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="inlineStr">
+        <is>
+          <t>Keramikkondensator 100 nF</t>
+        </is>
+      </c>
+      <c r="C48" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Keramikkondensator 100 nF",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D48" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="19" t="inlineStr">
+        <is>
+          <t>Hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="inlineStr">
+        <is>
+          <t>I2C-Hub / Multiplexer TCA9548A (optional)</t>
+        </is>
+      </c>
+      <c r="C49" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D49" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="19" t="inlineStr">
+        <is>
+          <t>nicht nötig, Platz vom Hub belegt</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="inlineStr">
+        <is>
+          <t>WS2812B-LED-Streifen (optional)</t>
+        </is>
+      </c>
+      <c r="C50" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"WS2812B-LED-Streifen (optional)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D50" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="19" t="inlineStr">
+        <is>
+          <t>Status-LEDs an IO4</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="inlineStr">
+        <is>
+          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
+        </is>
+      </c>
+      <c r="C51" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D51" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="19" t="inlineStr">
+        <is>
+          <t>Hub &lt;-&gt; Beine, Fußschalter, Taster, Treiber</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
+        </is>
+      </c>
+      <c r="C52" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D52" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E52" s="19" t="inlineStr">
+        <is>
+          <t>Servo-Anschlüsse Bein-Platinen</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
+        </is>
+      </c>
+      <c r="C53" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D53" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>Relais-Adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t>Dupont-Kabel (Trigger/Strobe)</t>
+        </is>
+      </c>
+      <c r="C54" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Dupont-Kabel (Trigger/Strobe)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D54" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="19" t="inlineStr">
+        <is>
+          <t>Kameras, I²C, Pi-GPIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>Servokabel 5264 3-pol.</t>
+        </is>
+      </c>
+      <c r="C55" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Servokabel 5264 3-pol.",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D55" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>H5 -&gt; Hub, ggf. Verlängerung</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B56" s="19" t="inlineStr">
+        <is>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
+        </is>
+      </c>
+      <c r="C56" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D56" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>gesteckte Signalleitungen</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B57" s="19" t="inlineStr">
+        <is>
+          <t>Litze AWG14 rot/schwarz (m)</t>
+        </is>
+      </c>
+      <c r="C57" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG14 rot/schwarz (m)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D57" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>Akku -&gt; F1 -&gt; Power-Board</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B58" s="19" t="inlineStr">
+        <is>
+          <t>Litze AWG20 rot/schwarz (m)</t>
+        </is>
+      </c>
+      <c r="C58" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG20 rot/schwarz (m)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D58" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E58" s="19" t="inlineStr">
+        <is>
+          <t>Strom je Bein, Relais, DC-DC, Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B59" s="19" t="inlineStr">
+        <is>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
+        </is>
+      </c>
+      <c r="C59" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D59" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E59" s="19" t="inlineStr">
+        <is>
+          <t>Sammelschienen Power-Board</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>Stecker &amp; Kabel</t>
+        </is>
+      </c>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
+        </is>
+      </c>
+      <c r="C60" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D60" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>Schienen Bein-Platinen, Hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>Platinen</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>Lochrasterplatinen AZ-Delivery</t>
+        </is>
+      </c>
+      <c r="C61" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Lochrasterplatinen AZ-Delivery",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D61" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>3× 3×7, 2× 5×7, 1× 2×8</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4666,7 +6199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5060,7 +6593,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fewer screw types: relay on inserts, one column length, M2x6 only
- Baseplate V2.11: relay bosses d8 with M3 insert pilot (4.0 x 6.5 from
  the top); relay fixed with M3x6 -> no M3x14, no nuts
- all 8 columns M3x50 (M3x45 dropped), lock nuts 10 (+4)
- M2x6 pan head (on hand) for camera and perfboards (M2x5 dropped)
- inserts, M2 screws and washers marked as on hand

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -635,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2199,11 +2199,11 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk; nicht länger</t>
+          <t>Gabelwange unten -&gt; Rückscheibe, 4 je Gelenk (72); Relaismodul in Gewindeeinsätze (4); nicht länger</t>
         </is>
       </c>
       <c r="E41" s="7" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F41" s="7" t="n">
         <v>8</v>
@@ -2273,11 +2273,11 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>6 Säulen unter den Panzersäulen, von unten in den Gewindeeinsatz</t>
+          <t>alle 8 Säulen von unten: 6 in die Gewindeeinsätze der Panzersäulen, 2 bei x = -40 mit Sicherungsmutter (5,6 mm Überstand unter dem Panzer)</t>
         </is>
       </c>
       <c r="E43" s="7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F43" s="7" t="n">
         <v>1</v>
@@ -2310,11 +2310,11 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>unten in den 6 Panzersäulen</t>
+          <t>Panzersäulen (6) + Relais-Bunde auf der unteren Platte (4)</t>
         </is>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F44" s="7" t="n">
         <v>2</v>
@@ -2328,7 +2328,11 @@
         <f>IF(H44="","",G44*H44)</f>
         <v/>
       </c>
-      <c r="J44" s="10" t="n"/>
+      <c r="J44" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K44" s="10" t="n"/>
     </row>
     <row r="45">
@@ -2342,16 +2346,16 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Zylinderschraube M3x12 + Mutter</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>2 Säulen bei x = -40 (mit Mutter, kein Panzerpfosten)</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
       <c r="E45" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45" s="7" t="n">
         <v>1</v>
@@ -2379,19 +2383,19 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12 + Mutter</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>Plattenstoß, 4 je Platte</t>
         </is>
       </c>
       <c r="E46" s="7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F46" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="3">
         <f>E46+F46</f>
@@ -2416,19 +2420,19 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß, 4 je Platte</t>
+          <t>Plattenstoß (8) + 2 Säulen M3x50 bei x = -40 (2)</t>
         </is>
       </c>
       <c r="E47" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F47" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G47" s="3">
         <f>E47+F47</f>
@@ -2453,19 +2457,19 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Zylinderschraube M3x10 + Mutter</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Plattenstoß (8) + 2 Säulen M3x45 (2) + Relais (4)</t>
+          <t>DC-DC-Laschen (2) + Hub-Träger (2) + Steckerhalter Akku (2) + Taster-Winkel (1)</t>
         </is>
       </c>
       <c r="E48" s="7" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F48" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G48" s="3">
         <f>E48+F48</f>
@@ -2490,19 +2494,19 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Linsenkopfschraube M2x6</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Relais auf 5-mm-Bolzen (alternativ M2x14)</t>
+          <t>Kamera-Platinen (8) + Lochraster-Platinen (18), direkt in die 1,7-mm-Kernlöcher</t>
         </is>
       </c>
       <c r="E49" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F49" s="7" t="n">
         <v>4</v>
-      </c>
-      <c r="F49" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="G49" s="3">
         <f>E49+F49</f>
@@ -2513,7 +2517,11 @@
         <f>IF(H49="","",G49*H49)</f>
         <v/>
       </c>
-      <c r="J49" s="10" t="n"/>
+      <c r="J49" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K49" s="10" t="n"/>
     </row>
     <row r="50">
@@ -2527,19 +2535,19 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10 + Mutter</t>
+          <t>Zylinderschraube M3x25 + Mutter</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>DC-DC-Laschen (2) + Hub-Träger (2) + Steckerhalter Akku (2) + Taster-Winkel (1)</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte (Bohrung 3,2 = M3)</t>
         </is>
       </c>
       <c r="E50" s="7" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F50" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G50" s="3">
         <f>E50+F50</f>
@@ -2564,16 +2572,16 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Zylinderschraube M2,5x16</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Kamera-Platinen, direkt ins 1,7-mm-Kernloch</t>
+          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
         </is>
       </c>
       <c r="E51" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F51" s="7" t="n">
         <v>2</v>
@@ -2601,19 +2609,19 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x5</t>
+          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Lochraster-Platinen: 6× Bein (je 2), Hub (4), Power-Verteiler (2), direkt ins 1,7-mm-Kernloch</t>
+          <t>liegen dem Treiber bei</t>
         </is>
       </c>
       <c r="E52" s="7" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="F52" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G52" s="3">
         <f>E52+F52</f>
@@ -2624,7 +2632,11 @@
         <f>IF(H52="","",G52*H52)</f>
         <v/>
       </c>
-      <c r="J52" s="10" t="n"/>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K52" s="10" t="n"/>
     </row>
     <row r="53">
@@ -2638,19 +2650,19 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x25 + Mutter</t>
+          <t>Zylinderschraube M2,5x5</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte (Bohrung 3,2 = M3)</t>
+          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
         </is>
       </c>
       <c r="E53" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F53" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="F53" s="7" t="n">
-        <v>1</v>
       </c>
       <c r="G53" s="3">
         <f>E53+F53</f>
@@ -2675,19 +2687,15 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x16</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Pi 5: von unten durch Platte, gedruckte Hülse und Pi in die Abstandsbolzen des AI HAT+ (ersetzt dessen lange Schrauben)</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n"/>
       <c r="E54" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F54" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G54" s="3">
         <f>E54+F54</f>
@@ -2698,7 +2706,11 @@
         <f>IF(H54="","",G54*H54)</f>
         <v/>
       </c>
-      <c r="J54" s="10" t="n"/>
+      <c r="J54" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K54" s="10" t="n"/>
     </row>
     <row r="55">
@@ -2712,16 +2724,16 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>liegen dem Treiber bei</t>
+          <t>Haltestifte Mikroschalter: quer durch Tibia und Schalterlöcher, bündig abknipsen (2 je Fuß); Ersatz: Stahlnagel Ø1,2 oder aufgebogene Büroklammer</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
-        <v>4</v>
+        <v>0.5</v>
       </c>
       <c r="F55" s="7" t="n">
         <v>0</v>
@@ -2735,11 +2747,7 @@
         <f>IF(H55="","",G55*H55)</f>
         <v/>
       </c>
-      <c r="J55" s="10" t="inlineStr">
-        <is>
-          <t>vorhanden</t>
-        </is>
-      </c>
+      <c r="J55" s="10" t="n"/>
       <c r="K55" s="10" t="n"/>
     </row>
     <row r="56">
@@ -2748,24 +2756,24 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E56" s="7" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="F56" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G56" s="3">
         <f>E56+F56</f>
@@ -2785,15 +2793,19 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="n"/>
+          <t>Klettband 20 mm (m)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+        </is>
+      </c>
       <c r="E57" s="7" t="n">
         <v>1</v>
       </c>
@@ -2818,21 +2830,21 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Haltestifte Mikroschalter: quer durch Tibia und Schalterlöcher, bündig abknipsen (2 je Fuß); Ersatz: Stahlnagel Ø1,2 oder aufgebogene Büroklammer</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F58" s="7" t="n">
         <v>0</v>
@@ -2860,16 +2872,16 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F59" s="7" t="n">
         <v>0</v>
@@ -2897,12 +2909,12 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
@@ -2929,21 +2941,21 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="7" t="n">
         <v>0</v>
@@ -2966,21 +2978,21 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="F62" s="7" t="n">
         <v>0</v>
@@ -3003,12 +3015,12 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>PLA orange (kg)</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -3017,7 +3029,7 @@
         </is>
       </c>
       <c r="E63" s="7" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="F63" s="7" t="n">
         <v>0</v>
@@ -3035,172 +3047,61 @@
       <c r="K63" s="10" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Filament</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>PETG schwarz (kg)</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F64" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" s="3">
-        <f>E64+F64</f>
-        <v/>
-      </c>
-      <c r="H64" s="8" t="n"/>
-      <c r="I64" s="9">
-        <f>IF(H64="","",G64*H64)</f>
-        <v/>
-      </c>
-      <c r="J64" s="10" t="n"/>
-      <c r="K64" s="10" t="n"/>
+      <c r="A64" s="3" t="n"/>
+      <c r="B64" s="3" t="n"/>
+      <c r="C64" s="3" t="n"/>
+      <c r="D64" s="3" t="n"/>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
+      <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
+      <c r="I64" s="3" t="n"/>
+      <c r="J64" s="3" t="n"/>
+      <c r="K64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>Filament</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>TPU 95A (kg)</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>Füße</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="F65" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G65" s="3">
-        <f>E65+F65</f>
-        <v/>
-      </c>
-      <c r="H65" s="8" t="n"/>
-      <c r="I65" s="9">
-        <f>IF(H65="","",G65*H65)</f>
-        <v/>
-      </c>
-      <c r="J65" s="10" t="n"/>
-      <c r="K65" s="10" t="n"/>
+      <c r="A65" s="3" t="n"/>
+      <c r="B65" s="3" t="n"/>
+      <c r="C65" s="3" t="n"/>
+      <c r="D65" s="3" t="n"/>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="3" t="n"/>
+      <c r="G65" s="3" t="n"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I65" s="11">
+        <f>SUM(I2:I63)</f>
+        <v/>
+      </c>
+      <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>Filament</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>PLA orange (kg)</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Zierleisten</t>
-        </is>
-      </c>
-      <c r="E66" s="7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F66" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G66" s="3">
-        <f>E66+F66</f>
-        <v/>
-      </c>
-      <c r="H66" s="8" t="n"/>
-      <c r="I66" s="9">
-        <f>IF(H66="","",G66*H66)</f>
-        <v/>
-      </c>
-      <c r="J66" s="10" t="n"/>
-      <c r="K66" s="10" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="n"/>
-      <c r="B67" s="3" t="n"/>
-      <c r="C67" s="3" t="n"/>
-      <c r="D67" s="3" t="n"/>
-      <c r="E67" s="3" t="n"/>
-      <c r="F67" s="3" t="n"/>
-      <c r="G67" s="3" t="n"/>
-      <c r="H67" s="3" t="n"/>
-      <c r="I67" s="3" t="n"/>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="3" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="n"/>
-      <c r="B68" s="3" t="n"/>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
-      <c r="G68" s="3" t="n"/>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I68" s="11">
-        <f>SUM(I2:I66)</f>
-        <v/>
-      </c>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="3" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="n"/>
-      <c r="B69" s="3" t="n"/>
-      <c r="C69" s="3" t="n"/>
-      <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="n"/>
-      <c r="F69" s="3" t="n"/>
-      <c r="G69" s="3" t="n"/>
-      <c r="H69" s="3" t="inlineStr">
+      <c r="A66" s="3" t="n"/>
+      <c r="B66" s="3" t="n"/>
+      <c r="C66" s="3" t="n"/>
+      <c r="D66" s="3" t="n"/>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="inlineStr">
         <is>
           <t>Preise erfasst</t>
         </is>
       </c>
-      <c r="I69" s="3">
-        <f>COUNT(H2:H66)&amp;" von 65"</f>
-        <v/>
-      </c>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="3" t="n"/>
+      <c r="I66" s="3">
+        <f>COUNT(H2:H63)&amp;" von 62"</f>
+        <v/>
+      </c>
+      <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3214,7 +3115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3299,45 +3200,45 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x5</t>
+          <t>Linsenkopfschraube M2x6</t>
         </is>
       </c>
       <c r="C6" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2x5",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Linsenkopfschraube M2x6",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D6" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x5",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Linsenkopfschraube M2x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Linsenkopfschraube M2x6",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Lochraster-Platinen in 1,7-mm-Kernlöcher</t>
+          <t>Kamera- und Lochraster-Platinen in 1,7-mm-Kernlöcher</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M2,5</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2x6</t>
+          <t>Zylinderschraube M2,5x5</t>
         </is>
       </c>
       <c r="C7" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2x6",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x5",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2x6",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Kamera-Platinen in 1,7-mm-Kernlöcher</t>
+          <t>Treiber auf Distanzhülsen (nur falls nicht beiliegend)</t>
         </is>
       </c>
     </row>
@@ -3349,45 +3250,45 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Zylinderschraube M2,5x16</t>
         </is>
       </c>
       <c r="C8" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x5",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x16",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D8" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Treiber auf Distanzhülsen (nur falls nicht beiliegend)</t>
+          <t>Pi 5 durch Platte + gedruckte Hülse in die HAT-Bolzen</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>M2,5</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x16</t>
+          <t>Zylinderschraube M3x6</t>
         </is>
       </c>
       <c r="C9" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x16",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x6",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D9" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Pi 5 durch Platte + gedruckte Hülse in die HAT-Bolzen</t>
+          <t>Gabelwange unten + Relaismodul (Gewindeeinsätze)</t>
         </is>
       </c>
     </row>
@@ -3399,20 +3300,20 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x6</t>
+          <t>Zylinderschraube M3x8</t>
         </is>
       </c>
       <c r="C10" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x6",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D10" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Gabelwange unten -&gt; Servo-Rückscheibe, 4 je Gelenk</t>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk</t>
         </is>
       </c>
     </row>
@@ -3424,20 +3325,17 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x8</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="C11" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D11" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10",Kaufteile!$G:$G)+SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D11" s="19" t="inlineStr"/>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk</t>
+          <t>Plattenstoß (8, mit Sicherungsmutter); DC-DC, Hub-Träger, Steckerhalter, Taster-Winkel (7, mit Mutter)</t>
         </is>
       </c>
     </row>
@@ -3449,17 +3347,20 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Zylinderschraube M3x12</t>
         </is>
       </c>
       <c r="C12" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10",Kaufteile!$G:$G)+SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10 + Mutter",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D12" s="19" t="inlineStr"/>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x12 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D12" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>Plattenstoß (8, mit Sicherungsmutter); DC-DC, Hub-Träger, Steckerhalter, Taster-Winkel (7, mit Mutter)</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
     </row>
@@ -3471,20 +3372,20 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12</t>
+          <t>Zylinderschraube M3x25</t>
         </is>
       </c>
       <c r="C13" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x12 + Mutter",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x25 + Mutter",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D13" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
     </row>
@@ -3496,277 +3397,277 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x14</t>
+          <t>Zylinderschraube M3x50</t>
         </is>
       </c>
       <c r="C14" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x14",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x50",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D14" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x14",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x14",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Relaismodul auf 5-mm-Bolzen</t>
+          <t>alle 8 Säulen (6 in Gewindeeinsätze, 2 mit Sicherungsmutter)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Muttern</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x25</t>
+          <t>Mutter M3 (DIN 934)</t>
         </is>
       </c>
       <c r="C15" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x25 + Mutter",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D15" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x*+ Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D15" s="19" t="inlineStr"/>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>zu allen Schrauben „+ Mutter“ (M3x10, M3x12, M3x25)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Muttern</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x45</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="C16" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x45",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Sicherungsmutter M3 (Nylonring)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D16" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x45",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x45",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>2 Säulen bei x = -40</t>
+          <t>Plattenstoß, 2 Säulen bei x = -40</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Einsätze</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x50</t>
+          <t>Gewindeeinsatz M3 (5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="C17" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x50",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D17" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>6 Säulen unter den Panzersäulen</t>
+          <t>Panzersäulen + Relais-Bunde</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Muttern</t>
+          <t>Sonstiges</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Mutter M3 (DIN 934)</t>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
         </is>
       </c>
       <c r="C18" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x*+ Mutter",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D18" s="19" t="inlineStr"/>
+        <f>SUMIF(Kaufteile!$C:$C,"Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D18" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>zu allen Schrauben „+ Mutter“ (M3x10, M3x12, M3x25)</t>
+          <t>Elektronik isoliert befestigen</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>Muttern</t>
+          <t>Sonstiges</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="C19" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Sicherungsmutter M3 (Nylonring)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Federstahldraht 1,2 mm (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D19" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t>Plattenstoß, Säulen M3x45, Relais</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>Einsätze</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Gewindeeinsatz M3 (5,7 lang, Ø4,6)</t>
-        </is>
-      </c>
-      <c r="C20" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D20" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>Panzersäulen</t>
-        </is>
-      </c>
-    </row>
+          <t>Haltestifte Mikroschalter</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
     <row r="21">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>Sonstiges</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="C21" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D21" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>Elektronik isoliert befestigen</t>
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Elektronik und Verdrahtung</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="19" t="inlineStr">
-        <is>
-          <t>Sonstiges</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
-        </is>
-      </c>
-      <c r="C22" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Federstahldraht 1,2 mm (m)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D22" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>Haltestifte Mikroschalter</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Gruppe</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Teil</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Bestellmenge</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Verwendung</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Antrieb</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>Servo ST3215 (Feetech/Waveshare, 12 V)</t>
+        </is>
+      </c>
+      <c r="C23" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D23" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>18 Servos, 3 je Bein</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>Elektronik und Verdrahtung</t>
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Rechner</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Raspberry Pi 5</t>
+        </is>
+      </c>
+      <c r="C24" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi 5",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D24" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>Perzeption, Planung</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Gruppe</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Teil</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Bestellmenge</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Verwendung</t>
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Rechner</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>Raspberry Pi Active Cooler</t>
+        </is>
+      </c>
+      <c r="C25" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi Active Cooler",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D25" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E25" s="19" t="inlineStr">
+        <is>
+          <t>falls nicht beim Pi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Antrieb</t>
+          <t>Rechner</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>Servo ST3215 (Feetech/Waveshare, 12 V)</t>
+          <t>Hailo-8 AI HAT+ (26 TOPS)</t>
         </is>
       </c>
       <c r="C26" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D26" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>18 Servos, 3 je Bein</t>
+          <t>NPU</t>
         </is>
       </c>
     </row>
@@ -3778,95 +3679,95 @@
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>Raspberry Pi 5</t>
+          <t>Waveshare General Driver for Robots</t>
         </is>
       </c>
       <c r="C27" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi 5",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Waveshare General Driver for Robots",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D27" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>Perzeption, Planung</t>
+          <t>ESP32, Servo-Bus</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="19" t="inlineStr">
         <is>
-          <t>Rechner</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>Raspberry Pi Active Cooler</t>
+          <t>LiPo ZEEE 3S 9000 mAh</t>
         </is>
       </c>
       <c r="C28" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi Active Cooler",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"LiPo ZEEE 3S 9000 mAh",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D28" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>falls nicht beim Pi</t>
+          <t>Akku</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>Rechner</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>Hailo-8 AI HAT+ (26 TOPS)</t>
+          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
         </is>
       </c>
       <c r="C29" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D29" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>NPU</t>
+          <t>Kurzschluss-, Überstrom-, Zellenschutz</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>Rechner</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Waveshare General Driver for Robots</t>
+          <t>Flachsicherung 30 A + Inline-Halter</t>
         </is>
       </c>
       <c r="C30" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Waveshare General Driver for Robots",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Flachsicherung 30 A + Inline-Halter",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D30" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>ESP32, Servo-Bus</t>
+          <t>F1 in der Plusleitung; Inline-Halter, Litze ≥ AWG14</t>
         </is>
       </c>
     </row>
@@ -3878,20 +3779,20 @@
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>LiPo ZEEE 3S 9000 mAh</t>
+          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
         </is>
       </c>
       <c r="C31" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"LiPo ZEEE 3S 9000 mAh",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D31" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>Akku</t>
+          <t>Steckerhalter</t>
         </is>
       </c>
     </row>
@@ -3903,20 +3804,20 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
+          <t>DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C</t>
         </is>
       </c>
       <c r="C32" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D32" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Kurzschluss-, Überstrom-, Zellenschutz</t>
+          <t>Pi-Versorgung</t>
         </is>
       </c>
     </row>
@@ -3928,95 +3829,95 @@
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>Flachsicherung 30 A + Inline-Halter</t>
+          <t>Relaismodul 8-Kanal</t>
         </is>
       </c>
       <c r="C33" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Flachsicherung 30 A + Inline-Halter",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Relaismodul 8-Kanal",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D33" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>F1 in der Plusleitung; Inline-Halter, Litze ≥ AWG14</t>
+          <t>K1 Pi, K2–K7 Beine</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Sensorik</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
+          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
         </is>
       </c>
       <c r="C34" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D34" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>Steckerhalter</t>
+          <t>Stereo</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Sensorik</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C</t>
+          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
         </is>
       </c>
       <c r="C35" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D35" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>Pi-Versorgung</t>
+          <t>Stereo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Sensorik</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>Relaismodul 8-Kanal</t>
+          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
         </is>
       </c>
       <c r="C36" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Relaismodul 8-Kanal",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D36" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>K1 Pi, K2–K7 Beine</t>
+          <t>Kamera -&gt; Pi</t>
         </is>
       </c>
     </row>
@@ -4028,20 +3929,20 @@
       </c>
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
+          <t>IMU ICM-20948 (Pimoroni-Breakout)</t>
         </is>
       </c>
       <c r="C37" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D37" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>Stereo</t>
+          <t>VIO/SLAM am Pi</t>
         </is>
       </c>
     </row>
@@ -4053,95 +3954,95 @@
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
+          <t>Mikroschalter D2F (oder ähnlich)</t>
         </is>
       </c>
       <c r="C38" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Mikroschalter D2F (oder ähnlich)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D38" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>Stereo</t>
+          <t>Fußkontakte</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="19" t="inlineStr">
         <is>
-          <t>Sensorik</t>
+          <t>Bauteile</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
+          <t>IO-Expander MCP23017-E (Modul/Breakout)</t>
         </is>
       </c>
       <c r="C39" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D39" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>Kamera -&gt; Pi</t>
+          <t>Hub-Platine</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>Sensorik</t>
+          <t>Bauteile</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>IMU ICM-20948 (Pimoroni-Breakout)</t>
+          <t>Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)</t>
         </is>
       </c>
       <c r="C40" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D40" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>VIO/SLAM am Pi</t>
+          <t>Ein/Aus</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>Sensorik</t>
+          <t>Bauteile</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>Mikroschalter D2F (oder ähnlich)</t>
+          <t>Widerstand 10 kΩ</t>
         </is>
       </c>
       <c r="C41" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Mikroschalter D2F (oder ähnlich)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 10 kΩ",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D41" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>Fußkontakte</t>
+          <t>Pull-ups Füße + Taster</t>
         </is>
       </c>
     </row>
@@ -4153,20 +4054,20 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>IO-Expander MCP23017-E (Modul/Breakout)</t>
+          <t>Widerstand 4,7 kΩ</t>
         </is>
       </c>
       <c r="C42" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 4,7 kΩ",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D42" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>Hub-Platine</t>
+          <t>Basiswiderstand BC547</t>
         </is>
       </c>
     </row>
@@ -4178,20 +4079,20 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)</t>
+          <t>Transistor BC547 (NPN)</t>
         </is>
       </c>
       <c r="C43" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Transistor BC547 (NPN)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D43" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>Ein/Aus</t>
+          <t>Relais-Adapter</t>
         </is>
       </c>
     </row>
@@ -4203,20 +4104,20 @@
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>Widerstand 10 kΩ</t>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
         </is>
       </c>
       <c r="C44" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 10 kΩ",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D44" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>Pull-ups Füße + Taster</t>
+          <t>Bein-Platinen</t>
         </is>
       </c>
     </row>
@@ -4228,145 +4129,145 @@
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>Widerstand 4,7 kΩ</t>
+          <t>Keramikkondensator 100 nF</t>
         </is>
       </c>
       <c r="C45" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 4,7 kΩ",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Keramikkondensator 100 nF",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D45" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>Basiswiderstand BC547</t>
+          <t>Hub</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>Bauteile</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>Transistor BC547 (NPN)</t>
+          <t>I2C-Hub / Multiplexer TCA9548A (optional)</t>
         </is>
       </c>
       <c r="C46" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Transistor BC547 (NPN)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D46" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>Relais-Adapter</t>
+          <t>nicht nötig, Platz vom Hub belegt</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>Bauteile</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
+          <t>WS2812B-LED-Streifen (optional)</t>
         </is>
       </c>
       <c r="C47" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"WS2812B-LED-Streifen (optional)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D47" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>Bein-Platinen</t>
+          <t>Status-LEDs an IO4</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="19" t="inlineStr">
         <is>
-          <t>Bauteile</t>
+          <t>Stecker &amp; Kabel</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>Keramikkondensator 100 nF</t>
+          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
         </is>
       </c>
       <c r="C48" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Keramikkondensator 100 nF",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D48" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>Hub</t>
+          <t>Hub &lt;-&gt; Beine, Fußschalter, Taster, Treiber</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="19" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Stecker &amp; Kabel</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>I2C-Hub / Multiplexer TCA9548A (optional)</t>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
         </is>
       </c>
       <c r="C49" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D49" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E49" s="19" t="inlineStr">
         <is>
-          <t>nicht nötig, Platz vom Hub belegt</t>
+          <t>Servo-Anschlüsse Bein-Platinen</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Stecker &amp; Kabel</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>WS2812B-LED-Streifen (optional)</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
         </is>
       </c>
       <c r="C50" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"WS2812B-LED-Streifen (optional)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D50" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>Status-LEDs an IO4</t>
+          <t>Relais-Adapter</t>
         </is>
       </c>
     </row>
@@ -4378,20 +4279,20 @@
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
+          <t>Dupont-Kabel (Trigger/Strobe)</t>
         </is>
       </c>
       <c r="C51" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Dupont-Kabel (Trigger/Strobe)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D51" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E51" s="19" t="inlineStr">
         <is>
-          <t>Hub &lt;-&gt; Beine, Fußschalter, Taster, Treiber</t>
+          <t>Kameras, I²C, Pi-GPIO</t>
         </is>
       </c>
     </row>
@@ -4403,20 +4304,20 @@
       </c>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
+          <t>Servokabel 5264 3-pol.</t>
         </is>
       </c>
       <c r="C52" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Servokabel 5264 3-pol.",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D52" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E52" s="19" t="inlineStr">
         <is>
-          <t>Servo-Anschlüsse Bein-Platinen</t>
+          <t>H5 -&gt; Hub, ggf. Verlängerung</t>
         </is>
       </c>
     </row>
@@ -4428,20 +4329,20 @@
       </c>
       <c r="B53" s="19" t="inlineStr">
         <is>
-          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
         </is>
       </c>
       <c r="C53" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D53" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E53" s="19" t="inlineStr">
         <is>
-          <t>Relais-Adapter</t>
+          <t>gesteckte Signalleitungen</t>
         </is>
       </c>
     </row>
@@ -4453,20 +4354,20 @@
       </c>
       <c r="B54" s="19" t="inlineStr">
         <is>
-          <t>Dupont-Kabel (Trigger/Strobe)</t>
+          <t>Litze AWG14 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="C54" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Dupont-Kabel (Trigger/Strobe)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG14 rot/schwarz (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D54" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E54" s="19" t="inlineStr">
         <is>
-          <t>Kameras, I²C, Pi-GPIO</t>
+          <t>Akku -&gt; F1 -&gt; Power-Board</t>
         </is>
       </c>
     </row>
@@ -4478,20 +4379,20 @@
       </c>
       <c r="B55" s="19" t="inlineStr">
         <is>
-          <t>Servokabel 5264 3-pol.</t>
+          <t>Litze AWG20 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="C55" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Servokabel 5264 3-pol.",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG20 rot/schwarz (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D55" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>H5 -&gt; Hub, ggf. Verlängerung</t>
+          <t>Strom je Bein, Relais, DC-DC, Pi</t>
         </is>
       </c>
     </row>
@@ -4503,20 +4404,20 @@
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
         </is>
       </c>
       <c r="C56" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D56" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>gesteckte Signalleitungen</t>
+          <t>Sammelschienen Power-Board</t>
         </is>
       </c>
     </row>
@@ -4528,118 +4429,43 @@
       </c>
       <c r="B57" s="19" t="inlineStr">
         <is>
-          <t>Litze AWG14 rot/schwarz (m)</t>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
         </is>
       </c>
       <c r="C57" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG14 rot/schwarz (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D57" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t>Akku -&gt; F1 -&gt; Power-Board</t>
+          <t>Schienen Bein-Platinen, Hub</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="19" t="inlineStr">
         <is>
-          <t>Stecker &amp; Kabel</t>
+          <t>Platinen</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
         <is>
-          <t>Litze AWG20 rot/schwarz (m)</t>
+          <t>Lochrasterplatinen AZ-Delivery</t>
         </is>
       </c>
       <c r="C58" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG20 rot/schwarz (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Lochrasterplatinen AZ-Delivery",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D58" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E58" s="19" t="inlineStr">
-        <is>
-          <t>Strom je Bein, Relais, DC-DC, Pi</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="19" t="inlineStr">
-        <is>
-          <t>Stecker &amp; Kabel</t>
-        </is>
-      </c>
-      <c r="B59" s="19" t="inlineStr">
-        <is>
-          <t>Kupferdraht 1,5 mm² massiv (m)</t>
-        </is>
-      </c>
-      <c r="C59" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D59" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E59" s="19" t="inlineStr">
-        <is>
-          <t>Sammelschienen Power-Board</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="19" t="inlineStr">
-        <is>
-          <t>Stecker &amp; Kabel</t>
-        </is>
-      </c>
-      <c r="B60" s="19" t="inlineStr">
-        <is>
-          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
-        </is>
-      </c>
-      <c r="C60" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D60" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E60" s="19" t="inlineStr">
-        <is>
-          <t>Schienen Bein-Platinen, Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="19" t="inlineStr">
-        <is>
-          <t>Platinen</t>
-        </is>
-      </c>
-      <c r="B61" s="19" t="inlineStr">
-        <is>
-          <t>Lochrasterplatinen AZ-Delivery</t>
-        </is>
-      </c>
-      <c r="C61" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Lochrasterplatinen AZ-Delivery",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D61" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E61" s="19" t="inlineStr">
         <is>
           <t>3× 3×7, 2× 5×7, 1× 2×8</t>
         </is>

</xml_diff>

<commit_message>
BOM: driver screws M2.5x7 are supplied, drop M2.5x5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185t9tPaxSFoR6YPk1eVvYK
</commit_message>
<xml_diff>
--- a/Drawings/Macros/SLARC_Stueckliste.xlsx
+++ b/Drawings/Macros/SLARC_Stueckliste.xlsx
@@ -635,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Distanzhülsen M2,5 x 16 (Treiber)</t>
+          <t>Distanzhülsen M2,5 x 16 + Schrauben M2,5x7 (Treiber)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -2650,19 +2650,15 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>Treiber-Distanzhülsen, falls keine Schrauben beiliegen</t>
-        </is>
-      </c>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n"/>
       <c r="E53" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G53" s="3">
         <f>E53+F53</f>
@@ -2673,7 +2669,11 @@
         <f>IF(H53="","",G53*H53)</f>
         <v/>
       </c>
-      <c r="J53" s="10" t="n"/>
+      <c r="J53" s="10" t="inlineStr">
+        <is>
+          <t>vorhanden</t>
+        </is>
+      </c>
       <c r="K53" s="10" t="n"/>
     </row>
     <row r="54">
@@ -2687,12 +2687,16 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="n"/>
+          <t>Federstahldraht 1,2 mm (m)</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Haltestifte Mikroschalter: quer durch Tibia und Schalterlöcher, bündig abknipsen (2 je Fuß); Ersatz: Stahlnagel Ø1,2 oder aufgebogene Büroklammer</t>
+        </is>
+      </c>
       <c r="E54" s="7" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F54" s="7" t="n">
         <v>0</v>
@@ -2706,11 +2710,7 @@
         <f>IF(H54="","",G54*H54)</f>
         <v/>
       </c>
-      <c r="J54" s="10" t="inlineStr">
-        <is>
-          <t>vorhanden</t>
-        </is>
-      </c>
+      <c r="J54" s="10" t="n"/>
       <c r="K54" s="10" t="n"/>
     </row>
     <row r="55">
@@ -2719,21 +2719,21 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Verbindung</t>
+          <t>Kleinteile</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
+          <t>Kabelbinder 2,5 mm</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Haltestifte Mikroschalter: quer durch Tibia und Schalterlöcher, bündig abknipsen (2 je Fuß); Ersatz: Stahlnagel Ø1,2 oder aufgebogene Büroklammer</t>
+          <t>Kabelösen Femur/Tibia</t>
         </is>
       </c>
       <c r="E55" s="7" t="n">
-        <v>0.5</v>
+        <v>50</v>
       </c>
       <c r="F55" s="7" t="n">
         <v>0</v>
@@ -2761,16 +2761,16 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Kabelbinder 2,5 mm</t>
+          <t>Klettband 20 mm (m)</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Kabelösen Femur/Tibia</t>
+          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
         </is>
       </c>
       <c r="E56" s="7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F56" s="7" t="n">
         <v>0</v>
@@ -2798,12 +2798,12 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Klettband 20 mm (m)</t>
+          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Batterie 2 Gurte, BMS 1 Gurt</t>
+          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
         </is>
       </c>
       <c r="E57" s="7" t="n">
@@ -2835,12 +2835,12 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Moosgummi EPDM 5 mm, selbstklebend (Streifen, ca. 20 mm breit)</t>
+          <t>Doppelseitiges Klebeband</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Akku: Streifen unter die obere Platte (Spalt 4,1 mm) gegen Klappern; 1 Stück 20x20 mit Ø9-Loch unter den Kopf des Akku-Riegels</t>
+          <t>Trigger-Platine</t>
         </is>
       </c>
       <c r="E58" s="7" t="n">
@@ -2872,12 +2872,12 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Doppelseitiges Klebeband</t>
+          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Trigger-Platine</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E59" s="7" t="n">
@@ -2904,21 +2904,21 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Kleinteile</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>2K-Epoxid oder Sekundenkleber + Primer</t>
+          <t>PETG schwarz (kg)</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Zierleisten</t>
+          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
         </is>
       </c>
       <c r="E60" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60" s="7" t="n">
         <v>0</v>
@@ -2946,16 +2946,16 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>PETG schwarz (kg)</t>
+          <t>TPU 95A (kg)</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>siehe Blatt Druckteile; inkl. Probedrucke</t>
+          <t>Füße</t>
         </is>
       </c>
       <c r="E61" s="7" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="F61" s="7" t="n">
         <v>0</v>
@@ -2983,16 +2983,16 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>TPU 95A (kg)</t>
+          <t>PLA orange (kg)</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Füße</t>
+          <t>Zierleisten</t>
         </is>
       </c>
       <c r="E62" s="7" t="n">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="F62" s="7" t="n">
         <v>0</v>
@@ -3010,41 +3010,17 @@
       <c r="K62" s="10" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>Filament</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>PLA orange (kg)</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>Zierleisten</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F63" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" s="3">
-        <f>E63+F63</f>
-        <v/>
-      </c>
-      <c r="H63" s="8" t="n"/>
-      <c r="I63" s="9">
-        <f>IF(H63="","",G63*H63)</f>
-        <v/>
-      </c>
-      <c r="J63" s="10" t="n"/>
-      <c r="K63" s="10" t="n"/>
+      <c r="A63" s="3" t="n"/>
+      <c r="B63" s="3" t="n"/>
+      <c r="C63" s="3" t="n"/>
+      <c r="D63" s="3" t="n"/>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
+      <c r="G63" s="3" t="n"/>
+      <c r="H63" s="3" t="n"/>
+      <c r="I63" s="3" t="n"/>
+      <c r="J63" s="3" t="n"/>
+      <c r="K63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -3054,8 +3030,15 @@
       <c r="E64" s="3" t="n"/>
       <c r="F64" s="3" t="n"/>
       <c r="G64" s="3" t="n"/>
-      <c r="H64" s="3" t="n"/>
-      <c r="I64" s="3" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Summe</t>
+        </is>
+      </c>
+      <c r="I64" s="11">
+        <f>SUM(I2:I62)</f>
+        <v/>
+      </c>
       <c r="J64" s="3" t="n"/>
       <c r="K64" s="3" t="n"/>
     </row>
@@ -3067,41 +3050,21 @@
       <c r="E65" s="3" t="n"/>
       <c r="F65" s="3" t="n"/>
       <c r="G65" s="3" t="n"/>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>Summe</t>
-        </is>
-      </c>
-      <c r="I65" s="11">
-        <f>SUM(I2:I63)</f>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Preise erfasst</t>
+        </is>
+      </c>
+      <c r="I65" s="3">
+        <f>COUNT(H2:H62)&amp;" von 61"</f>
         <v/>
       </c>
       <c r="J65" s="3" t="n"/>
       <c r="K65" s="3" t="n"/>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="n"/>
-      <c r="B66" s="3" t="n"/>
-      <c r="C66" s="3" t="n"/>
-      <c r="D66" s="3" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
-      <c r="G66" s="3" t="n"/>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>Preise erfasst</t>
-        </is>
-      </c>
-      <c r="I66" s="3">
-        <f>COUNT(H2:H63)&amp;" von 62"</f>
-        <v/>
-      </c>
-      <c r="J66" s="3" t="n"/>
-      <c r="K66" s="3" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bestellt,geliefert,vorhanden"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3115,7 +3078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3225,45 +3188,45 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x5</t>
+          <t>Zylinderschraube M2,5x16</t>
         </is>
       </c>
       <c r="C7" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x5",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x16",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D7" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x5",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Treiber auf Distanzhülsen (nur falls nicht beiliegend)</t>
+          <t>Pi 5 durch Platte + gedruckte Hülse in die HAT-Bolzen</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>M2,5</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M2,5x16</t>
+          <t>Zylinderschraube M3x6</t>
         </is>
       </c>
       <c r="C8" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M2,5x16",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x6",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D8" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M2,5x16",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Pi 5 durch Platte + gedruckte Hülse in die HAT-Bolzen</t>
+          <t>Gabelwange unten + Relaismodul (Gewindeeinsätze)</t>
         </is>
       </c>
     </row>
@@ -3275,20 +3238,20 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x6</t>
+          <t>Zylinderschraube M3x8</t>
         </is>
       </c>
       <c r="C9" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x6",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D9" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x6",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Gabelwange unten + Relaismodul (Gewindeeinsätze)</t>
+          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk</t>
         </is>
       </c>
     </row>
@@ -3300,20 +3263,17 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x8</t>
+          <t>Zylinderschraube M3x10</t>
         </is>
       </c>
       <c r="C10" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D10" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x8 (ISO 7380/4762)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10",Kaufteile!$G:$G)+SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D10" s="19" t="inlineStr"/>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Gabelwange oben -&gt; Horn, 4 je Gelenk</t>
+          <t>Plattenstoß (8, mit Sicherungsmutter); DC-DC, Hub-Träger, Steckerhalter, Taster-Winkel (7, mit Mutter)</t>
         </is>
       </c>
     </row>
@@ -3325,17 +3285,20 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x10</t>
+          <t>Zylinderschraube M3x12</t>
         </is>
       </c>
       <c r="C11" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10",Kaufteile!$G:$G)+SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x10 + Mutter",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D11" s="19" t="inlineStr"/>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x12 + Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D11" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>Plattenstoß (8, mit Sicherungsmutter); DC-DC, Hub-Träger, Steckerhalter, Taster-Winkel (7, mit Mutter)</t>
+          <t>Teilungsspant Panzer</t>
         </is>
       </c>
     </row>
@@ -3347,20 +3310,20 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x12</t>
+          <t>Zylinderschraube M3x25</t>
         </is>
       </c>
       <c r="C12" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x12 + Mutter",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x25 + Mutter",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D12" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x12 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>Teilungsspant Panzer</t>
+          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
         </is>
       </c>
     </row>
@@ -3372,45 +3335,42 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x25</t>
+          <t>Zylinderschraube M3x50</t>
         </is>
       </c>
       <c r="C13" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x25 + Mutter",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x50",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D13" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x25 + Mutter",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>Kamerahalter-Laschen durch Sockel + Platte</t>
+          <t>alle 8 Säulen (6 in Gewindeeinsätze, 2 mit Sicherungsmutter)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>Muttern</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Zylinderschraube M3x50</t>
+          <t>Mutter M3 (DIN 934)</t>
         </is>
       </c>
       <c r="C14" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x50",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D14" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Zylinderschraube M3x50",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
+        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x*+ Mutter",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D14" s="19" t="inlineStr"/>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>alle 8 Säulen (6 in Gewindeeinsätze, 2 mit Sicherungsmutter)</t>
+          <t>zu allen Schrauben „+ Mutter“ (M3x10, M3x12, M3x25)</t>
         </is>
       </c>
     </row>
@@ -3422,67 +3382,70 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Mutter M3 (DIN 934)</t>
+          <t>Sicherungsmutter M3 (Nylonring)</t>
         </is>
       </c>
       <c r="C15" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Zylinderschraube M3x*+ Mutter",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D15" s="19" t="inlineStr"/>
+        <f>SUMIF(Kaufteile!$C:$C,"Sicherungsmutter M3 (Nylonring)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D15" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>zu allen Schrauben „+ Mutter“ (M3x10, M3x12, M3x25)</t>
+          <t>Plattenstoß, 2 Säulen bei x = -40</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>Muttern</t>
+          <t>Einsätze</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Sicherungsmutter M3 (Nylonring)</t>
+          <t>Gewindeeinsatz M3 (5,7 lang, Ø4,6)</t>
         </is>
       </c>
       <c r="C16" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Sicherungsmutter M3 (Nylonring)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D16" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Sicherungsmutter M3 (Nylonring)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>Plattenstoß, 2 Säulen bei x = -40</t>
+          <t>Panzersäulen + Relais-Bunde</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Einsätze</t>
+          <t>Sonstiges</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Gewindeeinsatz M3 (5,7 lang, Ø4,6)</t>
+          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
         </is>
       </c>
       <c r="C17" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D17" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Gewindeeinsatz M3 (Einschmelzmutter, 5,7 lang, Ø4,6)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>Panzersäulen + Relais-Bunde</t>
+          <t>Elektronik isoliert befestigen</t>
         </is>
       </c>
     </row>
@@ -3494,105 +3457,105 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)</t>
+          <t>Federstahldraht 1,2 mm (m)</t>
         </is>
       </c>
       <c r="C18" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Federstahldraht 1,2 mm (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D18" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kunststoff-Unterlegscheiben M2/M2,5/M3 (Sortiment)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E18" s="19" t="inlineStr">
         <is>
-          <t>Elektronik isoliert befestigen</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>Sonstiges</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>Federstahldraht 1,2 mm (m)</t>
-        </is>
-      </c>
-      <c r="C19" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Federstahldraht 1,2 mm (m)",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D19" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Federstahldraht 1,2 mm (m)",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E19" s="19" t="inlineStr">
-        <is>
           <t>Haltestifte Mikroschalter</t>
         </is>
       </c>
     </row>
-    <row r="20"/>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Elektronik und Verdrahtung</t>
+        </is>
+      </c>
+    </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>Elektronik und Verdrahtung</t>
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Gruppe</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Teil</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Bestellmenge</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Verwendung</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Gruppe</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Teil</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Bestellmenge</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Verwendung</t>
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Antrieb</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Servo ST3215 (Feetech/Waveshare, 12 V)</t>
+        </is>
+      </c>
+      <c r="C22" s="19">
+        <f>SUMIF(Kaufteile!$C:$C,"Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$G:$G)</f>
+        <v/>
+      </c>
+      <c r="D22" s="19">
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))),"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>18 Servos, 3 je Bein</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>Antrieb</t>
+          <t>Rechner</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>Servo ST3215 (Feetech/Waveshare, 12 V)</t>
+          <t>Raspberry Pi 5</t>
         </is>
       </c>
       <c r="C23" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi 5",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D23" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servo ST3215 (Feetech/Waveshare, 12 V)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>18 Servos, 3 je Bein</t>
+          <t>Perzeption, Planung</t>
         </is>
       </c>
     </row>
@@ -3604,20 +3567,20 @@
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>Raspberry Pi 5</t>
+          <t>Raspberry Pi Active Cooler</t>
         </is>
       </c>
       <c r="C24" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi 5",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi Active Cooler",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D24" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi 5",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>Perzeption, Planung</t>
+          <t>falls nicht beim Pi</t>
         </is>
       </c>
     </row>
@@ -3629,20 +3592,20 @@
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>Raspberry Pi Active Cooler</t>
+          <t>Hailo-8 AI HAT+ (26 TOPS)</t>
         </is>
       </c>
       <c r="C25" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Raspberry Pi Active Cooler",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D25" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Raspberry Pi Active Cooler",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>falls nicht beim Pi</t>
+          <t>NPU</t>
         </is>
       </c>
     </row>
@@ -3654,45 +3617,45 @@
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>Hailo-8 AI HAT+ (26 TOPS)</t>
+          <t>Waveshare General Driver for Robots</t>
         </is>
       </c>
       <c r="C26" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Waveshare General Driver for Robots",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D26" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Hailo-8 AI HAT+ (26 TOPS)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>NPU</t>
+          <t>ESP32, Servo-Bus</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>Rechner</t>
+          <t>Energie</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>Waveshare General Driver for Robots</t>
+          <t>LiPo ZEEE 3S 9000 mAh</t>
         </is>
       </c>
       <c r="C27" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Waveshare General Driver for Robots",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"LiPo ZEEE 3S 9000 mAh",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D27" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Waveshare General Driver for Robots",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>ESP32, Servo-Bus</t>
+          <t>Akku</t>
         </is>
       </c>
     </row>
@@ -3704,20 +3667,20 @@
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>LiPo ZEEE 3S 9000 mAh</t>
+          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
         </is>
       </c>
       <c r="C28" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"LiPo ZEEE 3S 9000 mAh",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D28" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("LiPo ZEEE 3S 9000 mAh",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>Akku</t>
+          <t>Kurzschluss-, Überstrom-, Zellenschutz</t>
         </is>
       </c>
     </row>
@@ -3729,20 +3692,20 @@
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>BMS 3S (Daly 12 V 60 A oder 30–40 A)</t>
+          <t>Flachsicherung 30 A + Inline-Halter</t>
         </is>
       </c>
       <c r="C29" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Flachsicherung 30 A + Inline-Halter",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D29" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("BMS 3S (Daly 12 V 60 A oder 30–40 A)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>Kurzschluss-, Überstrom-, Zellenschutz</t>
+          <t>F1 in der Plusleitung; Inline-Halter, Litze ≥ AWG14</t>
         </is>
       </c>
     </row>
@@ -3754,20 +3717,20 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>Flachsicherung 30 A + Inline-Halter</t>
+          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
         </is>
       </c>
       <c r="C30" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Flachsicherung 30 A + Inline-Halter",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D30" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Flachsicherung 30 A + Inline-Halter",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>F1 in der Plusleitung; Inline-Halter, Litze ≥ AWG14</t>
+          <t>Steckerhalter</t>
         </is>
       </c>
     </row>
@@ -3779,20 +3742,20 @@
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Deans-T-Stecker (Stifte, Robot-Seite)</t>
+          <t>DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C</t>
         </is>
       </c>
       <c r="C31" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D31" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Deans-T-Stecker (Stifte, Robot-Seite)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>Steckerhalter</t>
+          <t>Pi-Versorgung</t>
         </is>
       </c>
     </row>
@@ -3804,45 +3767,45 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C</t>
+          <t>Relaismodul 8-Kanal</t>
         </is>
       </c>
       <c r="C32" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Relaismodul 8-Kanal",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D32" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("DC-DC 12 V -&gt; 5 V / 5 A Fulree F35J5V5A1S-C",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Pi-Versorgung</t>
+          <t>K1 Pi, K2–K7 Beine</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="19" t="inlineStr">
         <is>
-          <t>Energie</t>
+          <t>Sensorik</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>Relaismodul 8-Kanal</t>
+          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
         </is>
       </c>
       <c r="C33" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Relaismodul 8-Kanal",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D33" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Relaismodul 8-Kanal",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>K1 Pi, K2–K7 Beine</t>
+          <t>Stereo</t>
         </is>
       </c>
     </row>
@@ -3854,15 +3817,15 @@
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>IMX296 Kamera-Modul mit ext. Trigger</t>
+          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
         </is>
       </c>
       <c r="C34" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D34" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMX296 Kamera-Modul mit ext. Trigger",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -3879,20 +3842,20 @@
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>M12-Objektiv 2,8 mm (ZH3019-14)</t>
+          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
         </is>
       </c>
       <c r="C35" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D35" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("M12-Objektiv 2,8 mm (ZH3019-14)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>Stereo</t>
+          <t>Kamera -&gt; Pi</t>
         </is>
       </c>
     </row>
@@ -3904,20 +3867,20 @@
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm</t>
+          <t>IMU ICM-20948 (Pimoroni-Breakout)</t>
         </is>
       </c>
       <c r="C36" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D36" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("CSI-Kabel Pi 5 (22-pol auf 15-pol), ca. 200 mm",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>Kamera -&gt; Pi</t>
+          <t>VIO/SLAM am Pi</t>
         </is>
       </c>
     </row>
@@ -3929,45 +3892,45 @@
       </c>
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>IMU ICM-20948 (Pimoroni-Breakout)</t>
+          <t>Mikroschalter D2F (oder ähnlich)</t>
         </is>
       </c>
       <c r="C37" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Mikroschalter D2F (oder ähnlich)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D37" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IMU ICM-20948 (Pimoroni-Breakout)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>VIO/SLAM am Pi</t>
+          <t>Fußkontakte</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>Sensorik</t>
+          <t>Bauteile</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>Mikroschalter D2F (oder ähnlich)</t>
+          <t>IO-Expander MCP23017-E (Modul/Breakout)</t>
         </is>
       </c>
       <c r="C38" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Mikroschalter D2F (oder ähnlich)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D38" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Mikroschalter D2F (oder ähnlich)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>Fußkontakte</t>
+          <t>Hub-Platine</t>
         </is>
       </c>
     </row>
@@ -3979,20 +3942,20 @@
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>IO-Expander MCP23017-E (Modul/Breakout)</t>
+          <t>Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)</t>
         </is>
       </c>
       <c r="C39" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D39" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("IO-Expander MCP23017-E (Modul/Breakout)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>Hub-Platine</t>
+          <t>Ein/Aus</t>
         </is>
       </c>
     </row>
@@ -4004,20 +3967,20 @@
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)</t>
+          <t>Widerstand 10 kΩ</t>
         </is>
       </c>
       <c r="C40" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 10 kΩ",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D40" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Drucktaster 12 mm, Einbau, Schließer (Metall, IP65)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>Ein/Aus</t>
+          <t>Pull-ups Füße + Taster</t>
         </is>
       </c>
     </row>
@@ -4029,20 +3992,20 @@
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>Widerstand 10 kΩ</t>
+          <t>Widerstand 4,7 kΩ</t>
         </is>
       </c>
       <c r="C41" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 10 kΩ",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 4,7 kΩ",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D41" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 10 kΩ",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>Pull-ups Füße + Taster</t>
+          <t>Basiswiderstand BC547</t>
         </is>
       </c>
     </row>
@@ -4054,20 +4017,20 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>Widerstand 4,7 kΩ</t>
+          <t>Transistor BC547 (NPN)</t>
         </is>
       </c>
       <c r="C42" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Widerstand 4,7 kΩ",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Transistor BC547 (NPN)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D42" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Widerstand 4,7 kΩ",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>Basiswiderstand BC547</t>
+          <t>Relais-Adapter</t>
         </is>
       </c>
     </row>
@@ -4079,20 +4042,20 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>Transistor BC547 (NPN)</t>
+          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
         </is>
       </c>
       <c r="C43" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Transistor BC547 (NPN)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D43" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Transistor BC547 (NPN)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>Relais-Adapter</t>
+          <t>Bein-Platinen</t>
         </is>
       </c>
     </row>
@@ -4104,45 +4067,45 @@
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>Elko 470 µF / 25 V (radial, low ESR)</t>
+          <t>Keramikkondensator 100 nF</t>
         </is>
       </c>
       <c r="C44" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Keramikkondensator 100 nF",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D44" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Elko 470 µF / 25 V (radial, low ESR)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>Bein-Platinen</t>
+          <t>Hub</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>Bauteile</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>Keramikkondensator 100 nF</t>
+          <t>I2C-Hub / Multiplexer TCA9548A (optional)</t>
         </is>
       </c>
       <c r="C45" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Keramikkondensator 100 nF",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D45" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Keramikkondensator 100 nF",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>Hub</t>
+          <t>nicht nötig, Platz vom Hub belegt</t>
         </is>
       </c>
     </row>
@@ -4154,45 +4117,45 @@
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>I2C-Hub / Multiplexer TCA9548A (optional)</t>
+          <t>WS2812B-LED-Streifen (optional)</t>
         </is>
       </c>
       <c r="C46" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"WS2812B-LED-Streifen (optional)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D46" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("I2C-Hub / Multiplexer TCA9548A (optional)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>nicht nötig, Platz vom Hub belegt</t>
+          <t>Status-LEDs an IO4</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Stecker &amp; Kabel</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>WS2812B-LED-Streifen (optional)</t>
+          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
         </is>
       </c>
       <c r="C47" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"WS2812B-LED-Streifen (optional)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D47" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("WS2812B-LED-Streifen (optional)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>Status-LEDs an IO4</t>
+          <t>Hub &lt;-&gt; Beine, Fußschalter, Taster, Treiber</t>
         </is>
       </c>
     </row>
@@ -4204,20 +4167,20 @@
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>JST-XH 2,54 Steckverbinder-Sortiment</t>
+          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
         </is>
       </c>
       <c r="C48" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D48" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("JST-XH 2,54 Steckverbinder-Sortiment",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>Hub &lt;-&gt; Beine, Fußschalter, Taster, Treiber</t>
+          <t>Servo-Anschlüsse Bein-Platinen</t>
         </is>
       </c>
     </row>
@@ -4229,20 +4192,20 @@
       </c>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>Stiftleiste 2,54 mm gerade, 40-pol.</t>
+          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
         </is>
       </c>
       <c r="C49" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D49" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Stiftleiste 2,54 mm gerade, 40-pol.",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E49" s="19" t="inlineStr">
         <is>
-          <t>Servo-Anschlüsse Bein-Platinen</t>
+          <t>Relais-Adapter</t>
         </is>
       </c>
     </row>
@@ -4254,20 +4217,20 @@
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>Buchsenleiste 2,54 mm, 10-pol., gewinkelt</t>
+          <t>Dupont-Kabel (Trigger/Strobe)</t>
         </is>
       </c>
       <c r="C50" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Dupont-Kabel (Trigger/Strobe)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D50" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Buchsenleiste 2,54 mm, 10-pol., gewinkelt",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>Relais-Adapter</t>
+          <t>Kameras, I²C, Pi-GPIO</t>
         </is>
       </c>
     </row>
@@ -4279,20 +4242,20 @@
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>Dupont-Kabel (Trigger/Strobe)</t>
+          <t>Servokabel 5264 3-pol.</t>
         </is>
       </c>
       <c r="C51" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Dupont-Kabel (Trigger/Strobe)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Servokabel 5264 3-pol.",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D51" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Dupont-Kabel (Trigger/Strobe)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E51" s="19" t="inlineStr">
         <is>
-          <t>Kameras, I²C, Pi-GPIO</t>
+          <t>H5 -&gt; Hub, ggf. Verlängerung</t>
         </is>
       </c>
     </row>
@@ -4304,20 +4267,20 @@
       </c>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>Servokabel 5264 3-pol.</t>
+          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
         </is>
       </c>
       <c r="C52" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Servokabel 5264 3-pol.",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D52" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Servokabel 5264 3-pol.",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E52" s="19" t="inlineStr">
         <is>
-          <t>H5 -&gt; Hub, ggf. Verlängerung</t>
+          <t>gesteckte Signalleitungen</t>
         </is>
       </c>
     </row>
@@ -4329,20 +4292,20 @@
       </c>
       <c r="B53" s="19" t="inlineStr">
         <is>
-          <t>Signal-Litze AWG24, mehrere Farben (m)</t>
+          <t>Litze AWG14 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="C53" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG14 rot/schwarz (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D53" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Signal-Litze AWG24, mehrere Farben (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E53" s="19" t="inlineStr">
         <is>
-          <t>gesteckte Signalleitungen</t>
+          <t>Akku -&gt; F1 -&gt; Power-Board</t>
         </is>
       </c>
     </row>
@@ -4354,20 +4317,20 @@
       </c>
       <c r="B54" s="19" t="inlineStr">
         <is>
-          <t>Litze AWG14 rot/schwarz (m)</t>
+          <t>Litze AWG20 rot/schwarz (m)</t>
         </is>
       </c>
       <c r="C54" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG14 rot/schwarz (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG20 rot/schwarz (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D54" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG14 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E54" s="19" t="inlineStr">
         <is>
-          <t>Akku -&gt; F1 -&gt; Power-Board</t>
+          <t>Strom je Bein, Relais, DC-DC, Pi</t>
         </is>
       </c>
     </row>
@@ -4379,20 +4342,20 @@
       </c>
       <c r="B55" s="19" t="inlineStr">
         <is>
-          <t>Litze AWG20 rot/schwarz (m)</t>
+          <t>Kupferdraht 1,5 mm² massiv (m)</t>
         </is>
       </c>
       <c r="C55" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Litze AWG20 rot/schwarz (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D55" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Litze AWG20 rot/schwarz (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>Strom je Bein, Relais, DC-DC, Pi</t>
+          <t>Sammelschienen Power-Board</t>
         </is>
       </c>
     </row>
@@ -4404,68 +4367,43 @@
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>Kupferdraht 1,5 mm² massiv (m)</t>
+          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
         </is>
       </c>
       <c r="C56" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D56" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht 1,5 mm² massiv (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>Sammelschienen Power-Board</t>
+          <t>Schienen Bein-Platinen, Hub</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="19" t="inlineStr">
         <is>
-          <t>Stecker &amp; Kabel</t>
+          <t>Platinen</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
         <is>
-          <t>Kupferdraht verzinnt 0,8 mm (m)</t>
+          <t>Lochrasterplatinen AZ-Delivery</t>
         </is>
       </c>
       <c r="C57" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$G:$G)</f>
+        <f>SUMIF(Kaufteile!$C:$C,"Lochrasterplatinen AZ-Delivery",Kaufteile!$G:$G)</f>
         <v/>
       </c>
       <c r="D57" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Kupferdraht verzinnt 0,8 mm (m)",Kaufteile!$C:$C,0))),"")</f>
+        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))),"")</f>
         <v/>
       </c>
       <c r="E57" s="19" t="inlineStr">
-        <is>
-          <t>Schienen Bein-Platinen, Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="19" t="inlineStr">
-        <is>
-          <t>Platinen</t>
-        </is>
-      </c>
-      <c r="B58" s="19" t="inlineStr">
-        <is>
-          <t>Lochrasterplatinen AZ-Delivery</t>
-        </is>
-      </c>
-      <c r="C58" s="19">
-        <f>SUMIF(Kaufteile!$C:$C,"Lochrasterplatinen AZ-Delivery",Kaufteile!$G:$G)</f>
-        <v/>
-      </c>
-      <c r="D58" s="19">
-        <f>IFERROR(IF(INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))="","",INDEX(Kaufteile!$J:$J,MATCH("Lochrasterplatinen AZ-Delivery",Kaufteile!$C:$C,0))),"")</f>
-        <v/>
-      </c>
-      <c r="E58" s="19" t="inlineStr">
         <is>
           <t>3× 3×7, 2× 5×7, 1× 2×8</t>
         </is>

</xml_diff>